<commit_message>
Remove TCKNO column, add MÜSAİTLİK DURUMU column
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F2bKD8QwZtMnPmjESyq7MM
</commit_message>
<xml_diff>
--- a/DiscoverEU_KA155_Katilimci_Tablosu.xlsx
+++ b/DiscoverEU_KA155_Katilimci_Tablosu.xlsx
@@ -50,7 +50,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00B6D7A8"/>
-        <bgColor rgb="00B6D7A8"/>
       </patternFill>
     </fill>
   </fills>
@@ -80,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -89,6 +88,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -473,10 +475,10 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -508,22 +510,22 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>TCKNO</t>
+          <t>CİNSİYET</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>CİNSİYET</t>
+          <t>VİZE DURUMU</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>VİZE DURUMU</t>
+          <t>BİLET FİYATLARI</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>BİLET FİYATLARI</t>
+          <t>MÜSAİTLİK DURUMU</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -538,11 +540,11 @@
       <c r="C2" s="4" t="n"/>
       <c r="D2" s="2" t="n"/>
       <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
+      <c r="F2" s="2" t="n"/>
       <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="5" t="n"/>
-      <c r="J2" s="6" t="n"/>
+      <c r="H2" s="5" t="n"/>
+      <c r="I2" s="6" t="n"/>
+      <c r="J2" s="7" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n"/>
@@ -550,11 +552,11 @@
       <c r="C3" s="4" t="n"/>
       <c r="D3" s="2" t="n"/>
       <c r="E3" s="4" t="n"/>
-      <c r="F3" s="4" t="n"/>
+      <c r="F3" s="2" t="n"/>
       <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
-      <c r="I3" s="5" t="n"/>
-      <c r="J3" s="6" t="n"/>
+      <c r="H3" s="5" t="n"/>
+      <c r="I3" s="6" t="n"/>
+      <c r="J3" s="7" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n"/>
@@ -562,11 +564,11 @@
       <c r="C4" s="4" t="n"/>
       <c r="D4" s="2" t="n"/>
       <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
+      <c r="F4" s="2" t="n"/>
       <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="6" t="n"/>
+      <c r="H4" s="5" t="n"/>
+      <c r="I4" s="6" t="n"/>
+      <c r="J4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n"/>
@@ -574,11 +576,11 @@
       <c r="C5" s="4" t="n"/>
       <c r="D5" s="2" t="n"/>
       <c r="E5" s="4" t="n"/>
-      <c r="F5" s="4" t="n"/>
+      <c r="F5" s="2" t="n"/>
       <c r="G5" s="2" t="n"/>
-      <c r="H5" s="2" t="n"/>
-      <c r="I5" s="5" t="n"/>
-      <c r="J5" s="6" t="n"/>
+      <c r="H5" s="5" t="n"/>
+      <c r="I5" s="6" t="n"/>
+      <c r="J5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n"/>
@@ -586,11 +588,11 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="2" t="n"/>
       <c r="E6" s="4" t="n"/>
-      <c r="F6" s="4" t="n"/>
+      <c r="F6" s="2" t="n"/>
       <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="5" t="n"/>
-      <c r="J6" s="6" t="n"/>
+      <c r="H6" s="5" t="n"/>
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n"/>
@@ -598,11 +600,11 @@
       <c r="C7" s="4" t="n"/>
       <c r="D7" s="2" t="n"/>
       <c r="E7" s="4" t="n"/>
-      <c r="F7" s="4" t="n"/>
+      <c r="F7" s="2" t="n"/>
       <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" s="5" t="n"/>
-      <c r="J7" s="6" t="n"/>
+      <c r="H7" s="5" t="n"/>
+      <c r="I7" s="6" t="n"/>
+      <c r="J7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n"/>
@@ -610,11 +612,11 @@
       <c r="C8" s="4" t="n"/>
       <c r="D8" s="2" t="n"/>
       <c r="E8" s="4" t="n"/>
-      <c r="F8" s="4" t="n"/>
+      <c r="F8" s="2" t="n"/>
       <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="n"/>
-      <c r="I8" s="5" t="n"/>
-      <c r="J8" s="6" t="n"/>
+      <c r="H8" s="5" t="n"/>
+      <c r="I8" s="6" t="n"/>
+      <c r="J8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n"/>
@@ -622,11 +624,11 @@
       <c r="C9" s="4" t="n"/>
       <c r="D9" s="2" t="n"/>
       <c r="E9" s="4" t="n"/>
-      <c r="F9" s="4" t="n"/>
+      <c r="F9" s="2" t="n"/>
       <c r="G9" s="2" t="n"/>
-      <c r="H9" s="2" t="n"/>
-      <c r="I9" s="5" t="n"/>
-      <c r="J9" s="6" t="n"/>
+      <c r="H9" s="5" t="n"/>
+      <c r="I9" s="6" t="n"/>
+      <c r="J9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n"/>
@@ -634,11 +636,11 @@
       <c r="C10" s="4" t="n"/>
       <c r="D10" s="2" t="n"/>
       <c r="E10" s="4" t="n"/>
-      <c r="F10" s="4" t="n"/>
+      <c r="F10" s="2" t="n"/>
       <c r="G10" s="2" t="n"/>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="5" t="n"/>
-      <c r="J10" s="6" t="n"/>
+      <c r="H10" s="5" t="n"/>
+      <c r="I10" s="6" t="n"/>
+      <c r="J10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n"/>
@@ -646,11 +648,11 @@
       <c r="C11" s="4" t="n"/>
       <c r="D11" s="2" t="n"/>
       <c r="E11" s="4" t="n"/>
-      <c r="F11" s="4" t="n"/>
+      <c r="F11" s="2" t="n"/>
       <c r="G11" s="2" t="n"/>
-      <c r="H11" s="2" t="n"/>
-      <c r="I11" s="5" t="n"/>
-      <c r="J11" s="6" t="n"/>
+      <c r="H11" s="5" t="n"/>
+      <c r="I11" s="6" t="n"/>
+      <c r="J11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n"/>
@@ -658,11 +660,11 @@
       <c r="C12" s="4" t="n"/>
       <c r="D12" s="2" t="n"/>
       <c r="E12" s="4" t="n"/>
-      <c r="F12" s="4" t="n"/>
+      <c r="F12" s="2" t="n"/>
       <c r="G12" s="2" t="n"/>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="5" t="n"/>
-      <c r="J12" s="6" t="n"/>
+      <c r="H12" s="5" t="n"/>
+      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n"/>
@@ -670,11 +672,11 @@
       <c r="C13" s="4" t="n"/>
       <c r="D13" s="2" t="n"/>
       <c r="E13" s="4" t="n"/>
-      <c r="F13" s="4" t="n"/>
+      <c r="F13" s="2" t="n"/>
       <c r="G13" s="2" t="n"/>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="5" t="n"/>
-      <c r="J13" s="6" t="n"/>
+      <c r="H13" s="5" t="n"/>
+      <c r="I13" s="6" t="n"/>
+      <c r="J13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n"/>
@@ -682,11 +684,11 @@
       <c r="C14" s="4" t="n"/>
       <c r="D14" s="2" t="n"/>
       <c r="E14" s="4" t="n"/>
-      <c r="F14" s="4" t="n"/>
+      <c r="F14" s="2" t="n"/>
       <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="5" t="n"/>
-      <c r="J14" s="6" t="n"/>
+      <c r="H14" s="5" t="n"/>
+      <c r="I14" s="6" t="n"/>
+      <c r="J14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n"/>
@@ -694,11 +696,11 @@
       <c r="C15" s="4" t="n"/>
       <c r="D15" s="2" t="n"/>
       <c r="E15" s="4" t="n"/>
-      <c r="F15" s="4" t="n"/>
+      <c r="F15" s="2" t="n"/>
       <c r="G15" s="2" t="n"/>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="5" t="n"/>
-      <c r="J15" s="6" t="n"/>
+      <c r="H15" s="5" t="n"/>
+      <c r="I15" s="6" t="n"/>
+      <c r="J15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n"/>
@@ -706,11 +708,11 @@
       <c r="C16" s="4" t="n"/>
       <c r="D16" s="2" t="n"/>
       <c r="E16" s="4" t="n"/>
-      <c r="F16" s="4" t="n"/>
+      <c r="F16" s="2" t="n"/>
       <c r="G16" s="2" t="n"/>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="5" t="n"/>
-      <c r="J16" s="6" t="n"/>
+      <c r="H16" s="5" t="n"/>
+      <c r="I16" s="6" t="n"/>
+      <c r="J16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n"/>
@@ -718,11 +720,11 @@
       <c r="C17" s="4" t="n"/>
       <c r="D17" s="2" t="n"/>
       <c r="E17" s="4" t="n"/>
-      <c r="F17" s="4" t="n"/>
+      <c r="F17" s="2" t="n"/>
       <c r="G17" s="2" t="n"/>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="5" t="n"/>
-      <c r="J17" s="6" t="n"/>
+      <c r="H17" s="5" t="n"/>
+      <c r="I17" s="6" t="n"/>
+      <c r="J17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n"/>
@@ -730,11 +732,11 @@
       <c r="C18" s="4" t="n"/>
       <c r="D18" s="2" t="n"/>
       <c r="E18" s="4" t="n"/>
-      <c r="F18" s="4" t="n"/>
+      <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="n"/>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="5" t="n"/>
-      <c r="J18" s="6" t="n"/>
+      <c r="H18" s="5" t="n"/>
+      <c r="I18" s="6" t="n"/>
+      <c r="J18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n"/>
@@ -742,11 +744,11 @@
       <c r="C19" s="4" t="n"/>
       <c r="D19" s="2" t="n"/>
       <c r="E19" s="4" t="n"/>
-      <c r="F19" s="4" t="n"/>
+      <c r="F19" s="2" t="n"/>
       <c r="G19" s="2" t="n"/>
-      <c r="H19" s="2" t="n"/>
-      <c r="I19" s="5" t="n"/>
-      <c r="J19" s="6" t="n"/>
+      <c r="H19" s="5" t="n"/>
+      <c r="I19" s="6" t="n"/>
+      <c r="J19" s="7" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n"/>
@@ -754,11 +756,11 @@
       <c r="C20" s="4" t="n"/>
       <c r="D20" s="2" t="n"/>
       <c r="E20" s="4" t="n"/>
-      <c r="F20" s="4" t="n"/>
+      <c r="F20" s="2" t="n"/>
       <c r="G20" s="2" t="n"/>
-      <c r="H20" s="2" t="n"/>
-      <c r="I20" s="5" t="n"/>
-      <c r="J20" s="6" t="n"/>
+      <c r="H20" s="5" t="n"/>
+      <c r="I20" s="6" t="n"/>
+      <c r="J20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n"/>
@@ -766,11 +768,11 @@
       <c r="C21" s="4" t="n"/>
       <c r="D21" s="2" t="n"/>
       <c r="E21" s="4" t="n"/>
-      <c r="F21" s="4" t="n"/>
+      <c r="F21" s="2" t="n"/>
       <c r="G21" s="2" t="n"/>
-      <c r="H21" s="2" t="n"/>
-      <c r="I21" s="5" t="n"/>
-      <c r="J21" s="6" t="n"/>
+      <c r="H21" s="5" t="n"/>
+      <c r="I21" s="6" t="n"/>
+      <c r="J21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n"/>
@@ -778,11 +780,11 @@
       <c r="C22" s="4" t="n"/>
       <c r="D22" s="2" t="n"/>
       <c r="E22" s="4" t="n"/>
-      <c r="F22" s="4" t="n"/>
+      <c r="F22" s="2" t="n"/>
       <c r="G22" s="2" t="n"/>
-      <c r="H22" s="2" t="n"/>
-      <c r="I22" s="5" t="n"/>
-      <c r="J22" s="6" t="n"/>
+      <c r="H22" s="5" t="n"/>
+      <c r="I22" s="6" t="n"/>
+      <c r="J22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n"/>
@@ -790,11 +792,11 @@
       <c r="C23" s="4" t="n"/>
       <c r="D23" s="2" t="n"/>
       <c r="E23" s="4" t="n"/>
-      <c r="F23" s="4" t="n"/>
+      <c r="F23" s="2" t="n"/>
       <c r="G23" s="2" t="n"/>
-      <c r="H23" s="2" t="n"/>
-      <c r="I23" s="5" t="n"/>
-      <c r="J23" s="6" t="n"/>
+      <c r="H23" s="5" t="n"/>
+      <c r="I23" s="6" t="n"/>
+      <c r="J23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n"/>
@@ -802,11 +804,11 @@
       <c r="C24" s="4" t="n"/>
       <c r="D24" s="2" t="n"/>
       <c r="E24" s="4" t="n"/>
-      <c r="F24" s="4" t="n"/>
+      <c r="F24" s="2" t="n"/>
       <c r="G24" s="2" t="n"/>
-      <c r="H24" s="2" t="n"/>
-      <c r="I24" s="5" t="n"/>
-      <c r="J24" s="6" t="n"/>
+      <c r="H24" s="5" t="n"/>
+      <c r="I24" s="6" t="n"/>
+      <c r="J24" s="7" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n"/>
@@ -814,11 +816,11 @@
       <c r="C25" s="4" t="n"/>
       <c r="D25" s="2" t="n"/>
       <c r="E25" s="4" t="n"/>
-      <c r="F25" s="4" t="n"/>
+      <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="n"/>
-      <c r="H25" s="2" t="n"/>
-      <c r="I25" s="5" t="n"/>
-      <c r="J25" s="6" t="n"/>
+      <c r="H25" s="5" t="n"/>
+      <c r="I25" s="6" t="n"/>
+      <c r="J25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n"/>
@@ -826,11 +828,11 @@
       <c r="C26" s="4" t="n"/>
       <c r="D26" s="2" t="n"/>
       <c r="E26" s="4" t="n"/>
-      <c r="F26" s="4" t="n"/>
+      <c r="F26" s="2" t="n"/>
       <c r="G26" s="2" t="n"/>
-      <c r="H26" s="2" t="n"/>
-      <c r="I26" s="5" t="n"/>
-      <c r="J26" s="6" t="n"/>
+      <c r="H26" s="5" t="n"/>
+      <c r="I26" s="6" t="n"/>
+      <c r="J26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n"/>
@@ -838,11 +840,11 @@
       <c r="C27" s="4" t="n"/>
       <c r="D27" s="2" t="n"/>
       <c r="E27" s="4" t="n"/>
-      <c r="F27" s="4" t="n"/>
+      <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="n"/>
-      <c r="H27" s="2" t="n"/>
-      <c r="I27" s="5" t="n"/>
-      <c r="J27" s="6" t="n"/>
+      <c r="H27" s="5" t="n"/>
+      <c r="I27" s="6" t="n"/>
+      <c r="J27" s="7" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n"/>
@@ -850,11 +852,11 @@
       <c r="C28" s="4" t="n"/>
       <c r="D28" s="2" t="n"/>
       <c r="E28" s="4" t="n"/>
-      <c r="F28" s="4" t="n"/>
+      <c r="F28" s="2" t="n"/>
       <c r="G28" s="2" t="n"/>
-      <c r="H28" s="2" t="n"/>
-      <c r="I28" s="5" t="n"/>
-      <c r="J28" s="6" t="n"/>
+      <c r="H28" s="5" t="n"/>
+      <c r="I28" s="6" t="n"/>
+      <c r="J28" s="7" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n"/>
@@ -862,11 +864,11 @@
       <c r="C29" s="4" t="n"/>
       <c r="D29" s="2" t="n"/>
       <c r="E29" s="4" t="n"/>
-      <c r="F29" s="4" t="n"/>
+      <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="n"/>
-      <c r="H29" s="2" t="n"/>
-      <c r="I29" s="5" t="n"/>
-      <c r="J29" s="6" t="n"/>
+      <c r="H29" s="5" t="n"/>
+      <c r="I29" s="6" t="n"/>
+      <c r="J29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n"/>
@@ -874,11 +876,11 @@
       <c r="C30" s="4" t="n"/>
       <c r="D30" s="2" t="n"/>
       <c r="E30" s="4" t="n"/>
-      <c r="F30" s="4" t="n"/>
+      <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="n"/>
-      <c r="H30" s="2" t="n"/>
-      <c r="I30" s="5" t="n"/>
-      <c r="J30" s="6" t="n"/>
+      <c r="H30" s="5" t="n"/>
+      <c r="I30" s="6" t="n"/>
+      <c r="J30" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n"/>
@@ -886,11 +888,11 @@
       <c r="C31" s="4" t="n"/>
       <c r="D31" s="2" t="n"/>
       <c r="E31" s="4" t="n"/>
-      <c r="F31" s="4" t="n"/>
+      <c r="F31" s="2" t="n"/>
       <c r="G31" s="2" t="n"/>
-      <c r="H31" s="2" t="n"/>
-      <c r="I31" s="5" t="n"/>
-      <c r="J31" s="6" t="n"/>
+      <c r="H31" s="5" t="n"/>
+      <c r="I31" s="6" t="n"/>
+      <c r="J31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n"/>
@@ -898,11 +900,11 @@
       <c r="C32" s="4" t="n"/>
       <c r="D32" s="2" t="n"/>
       <c r="E32" s="4" t="n"/>
-      <c r="F32" s="4" t="n"/>
+      <c r="F32" s="2" t="n"/>
       <c r="G32" s="2" t="n"/>
-      <c r="H32" s="2" t="n"/>
-      <c r="I32" s="5" t="n"/>
-      <c r="J32" s="6" t="n"/>
+      <c r="H32" s="5" t="n"/>
+      <c r="I32" s="6" t="n"/>
+      <c r="J32" s="7" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n"/>
@@ -910,11 +912,11 @@
       <c r="C33" s="4" t="n"/>
       <c r="D33" s="2" t="n"/>
       <c r="E33" s="4" t="n"/>
-      <c r="F33" s="4" t="n"/>
+      <c r="F33" s="2" t="n"/>
       <c r="G33" s="2" t="n"/>
-      <c r="H33" s="2" t="n"/>
-      <c r="I33" s="5" t="n"/>
-      <c r="J33" s="6" t="n"/>
+      <c r="H33" s="5" t="n"/>
+      <c r="I33" s="6" t="n"/>
+      <c r="J33" s="7" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n"/>
@@ -922,11 +924,11 @@
       <c r="C34" s="4" t="n"/>
       <c r="D34" s="2" t="n"/>
       <c r="E34" s="4" t="n"/>
-      <c r="F34" s="4" t="n"/>
+      <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="n"/>
-      <c r="H34" s="2" t="n"/>
-      <c r="I34" s="5" t="n"/>
-      <c r="J34" s="6" t="n"/>
+      <c r="H34" s="5" t="n"/>
+      <c r="I34" s="6" t="n"/>
+      <c r="J34" s="7" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n"/>
@@ -934,11 +936,11 @@
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="2" t="n"/>
       <c r="E35" s="4" t="n"/>
-      <c r="F35" s="4" t="n"/>
+      <c r="F35" s="2" t="n"/>
       <c r="G35" s="2" t="n"/>
-      <c r="H35" s="2" t="n"/>
-      <c r="I35" s="5" t="n"/>
-      <c r="J35" s="6" t="n"/>
+      <c r="H35" s="5" t="n"/>
+      <c r="I35" s="6" t="n"/>
+      <c r="J35" s="7" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n"/>
@@ -946,11 +948,11 @@
       <c r="C36" s="4" t="n"/>
       <c r="D36" s="2" t="n"/>
       <c r="E36" s="4" t="n"/>
-      <c r="F36" s="4" t="n"/>
+      <c r="F36" s="2" t="n"/>
       <c r="G36" s="2" t="n"/>
-      <c r="H36" s="2" t="n"/>
-      <c r="I36" s="5" t="n"/>
-      <c r="J36" s="6" t="n"/>
+      <c r="H36" s="5" t="n"/>
+      <c r="I36" s="6" t="n"/>
+      <c r="J36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n"/>
@@ -958,11 +960,11 @@
       <c r="C37" s="4" t="n"/>
       <c r="D37" s="2" t="n"/>
       <c r="E37" s="4" t="n"/>
-      <c r="F37" s="4" t="n"/>
+      <c r="F37" s="2" t="n"/>
       <c r="G37" s="2" t="n"/>
-      <c r="H37" s="2" t="n"/>
-      <c r="I37" s="5" t="n"/>
-      <c r="J37" s="6" t="n"/>
+      <c r="H37" s="5" t="n"/>
+      <c r="I37" s="6" t="n"/>
+      <c r="J37" s="7" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n"/>
@@ -970,11 +972,11 @@
       <c r="C38" s="4" t="n"/>
       <c r="D38" s="2" t="n"/>
       <c r="E38" s="4" t="n"/>
-      <c r="F38" s="4" t="n"/>
+      <c r="F38" s="2" t="n"/>
       <c r="G38" s="2" t="n"/>
-      <c r="H38" s="2" t="n"/>
-      <c r="I38" s="5" t="n"/>
-      <c r="J38" s="6" t="n"/>
+      <c r="H38" s="5" t="n"/>
+      <c r="I38" s="6" t="n"/>
+      <c r="J38" s="7" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n"/>
@@ -982,11 +984,11 @@
       <c r="C39" s="4" t="n"/>
       <c r="D39" s="2" t="n"/>
       <c r="E39" s="4" t="n"/>
-      <c r="F39" s="4" t="n"/>
+      <c r="F39" s="2" t="n"/>
       <c r="G39" s="2" t="n"/>
-      <c r="H39" s="2" t="n"/>
-      <c r="I39" s="5" t="n"/>
-      <c r="J39" s="6" t="n"/>
+      <c r="H39" s="5" t="n"/>
+      <c r="I39" s="6" t="n"/>
+      <c r="J39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n"/>
@@ -994,11 +996,11 @@
       <c r="C40" s="4" t="n"/>
       <c r="D40" s="2" t="n"/>
       <c r="E40" s="4" t="n"/>
-      <c r="F40" s="4" t="n"/>
+      <c r="F40" s="2" t="n"/>
       <c r="G40" s="2" t="n"/>
-      <c r="H40" s="2" t="n"/>
-      <c r="I40" s="5" t="n"/>
-      <c r="J40" s="6" t="n"/>
+      <c r="H40" s="5" t="n"/>
+      <c r="I40" s="6" t="n"/>
+      <c r="J40" s="7" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n"/>
@@ -1006,11 +1008,11 @@
       <c r="C41" s="4" t="n"/>
       <c r="D41" s="2" t="n"/>
       <c r="E41" s="4" t="n"/>
-      <c r="F41" s="4" t="n"/>
+      <c r="F41" s="2" t="n"/>
       <c r="G41" s="2" t="n"/>
-      <c r="H41" s="2" t="n"/>
-      <c r="I41" s="5" t="n"/>
-      <c r="J41" s="6" t="n"/>
+      <c r="H41" s="5" t="n"/>
+      <c r="I41" s="6" t="n"/>
+      <c r="J41" s="7" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n"/>
@@ -1018,11 +1020,11 @@
       <c r="C42" s="4" t="n"/>
       <c r="D42" s="2" t="n"/>
       <c r="E42" s="4" t="n"/>
-      <c r="F42" s="4" t="n"/>
+      <c r="F42" s="2" t="n"/>
       <c r="G42" s="2" t="n"/>
-      <c r="H42" s="2" t="n"/>
-      <c r="I42" s="5" t="n"/>
-      <c r="J42" s="6" t="n"/>
+      <c r="H42" s="5" t="n"/>
+      <c r="I42" s="6" t="n"/>
+      <c r="J42" s="7" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n"/>
@@ -1030,11 +1032,11 @@
       <c r="C43" s="4" t="n"/>
       <c r="D43" s="2" t="n"/>
       <c r="E43" s="4" t="n"/>
-      <c r="F43" s="4" t="n"/>
+      <c r="F43" s="2" t="n"/>
       <c r="G43" s="2" t="n"/>
-      <c r="H43" s="2" t="n"/>
-      <c r="I43" s="5" t="n"/>
-      <c r="J43" s="6" t="n"/>
+      <c r="H43" s="5" t="n"/>
+      <c r="I43" s="6" t="n"/>
+      <c r="J43" s="7" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n"/>
@@ -1042,11 +1044,11 @@
       <c r="C44" s="4" t="n"/>
       <c r="D44" s="2" t="n"/>
       <c r="E44" s="4" t="n"/>
-      <c r="F44" s="4" t="n"/>
+      <c r="F44" s="2" t="n"/>
       <c r="G44" s="2" t="n"/>
-      <c r="H44" s="2" t="n"/>
-      <c r="I44" s="5" t="n"/>
-      <c r="J44" s="6" t="n"/>
+      <c r="H44" s="5" t="n"/>
+      <c r="I44" s="6" t="n"/>
+      <c r="J44" s="7" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n"/>
@@ -1054,11 +1056,11 @@
       <c r="C45" s="4" t="n"/>
       <c r="D45" s="2" t="n"/>
       <c r="E45" s="4" t="n"/>
-      <c r="F45" s="4" t="n"/>
+      <c r="F45" s="2" t="n"/>
       <c r="G45" s="2" t="n"/>
-      <c r="H45" s="2" t="n"/>
-      <c r="I45" s="5" t="n"/>
-      <c r="J45" s="6" t="n"/>
+      <c r="H45" s="5" t="n"/>
+      <c r="I45" s="6" t="n"/>
+      <c r="J45" s="7" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n"/>
@@ -1066,11 +1068,11 @@
       <c r="C46" s="4" t="n"/>
       <c r="D46" s="2" t="n"/>
       <c r="E46" s="4" t="n"/>
-      <c r="F46" s="4" t="n"/>
+      <c r="F46" s="2" t="n"/>
       <c r="G46" s="2" t="n"/>
-      <c r="H46" s="2" t="n"/>
-      <c r="I46" s="5" t="n"/>
-      <c r="J46" s="6" t="n"/>
+      <c r="H46" s="5" t="n"/>
+      <c r="I46" s="6" t="n"/>
+      <c r="J46" s="7" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n"/>
@@ -1078,11 +1080,11 @@
       <c r="C47" s="4" t="n"/>
       <c r="D47" s="2" t="n"/>
       <c r="E47" s="4" t="n"/>
-      <c r="F47" s="4" t="n"/>
+      <c r="F47" s="2" t="n"/>
       <c r="G47" s="2" t="n"/>
-      <c r="H47" s="2" t="n"/>
-      <c r="I47" s="5" t="n"/>
-      <c r="J47" s="6" t="n"/>
+      <c r="H47" s="5" t="n"/>
+      <c r="I47" s="6" t="n"/>
+      <c r="J47" s="7" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n"/>
@@ -1090,11 +1092,11 @@
       <c r="C48" s="4" t="n"/>
       <c r="D48" s="2" t="n"/>
       <c r="E48" s="4" t="n"/>
-      <c r="F48" s="4" t="n"/>
+      <c r="F48" s="2" t="n"/>
       <c r="G48" s="2" t="n"/>
-      <c r="H48" s="2" t="n"/>
-      <c r="I48" s="5" t="n"/>
-      <c r="J48" s="6" t="n"/>
+      <c r="H48" s="5" t="n"/>
+      <c r="I48" s="6" t="n"/>
+      <c r="J48" s="7" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n"/>
@@ -1102,11 +1104,11 @@
       <c r="C49" s="4" t="n"/>
       <c r="D49" s="2" t="n"/>
       <c r="E49" s="4" t="n"/>
-      <c r="F49" s="4" t="n"/>
+      <c r="F49" s="2" t="n"/>
       <c r="G49" s="2" t="n"/>
-      <c r="H49" s="2" t="n"/>
-      <c r="I49" s="5" t="n"/>
-      <c r="J49" s="6" t="n"/>
+      <c r="H49" s="5" t="n"/>
+      <c r="I49" s="6" t="n"/>
+      <c r="J49" s="7" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n"/>
@@ -1114,11 +1116,11 @@
       <c r="C50" s="4" t="n"/>
       <c r="D50" s="2" t="n"/>
       <c r="E50" s="4" t="n"/>
-      <c r="F50" s="4" t="n"/>
+      <c r="F50" s="2" t="n"/>
       <c r="G50" s="2" t="n"/>
-      <c r="H50" s="2" t="n"/>
-      <c r="I50" s="5" t="n"/>
-      <c r="J50" s="6" t="n"/>
+      <c r="H50" s="5" t="n"/>
+      <c r="I50" s="6" t="n"/>
+      <c r="J50" s="7" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n"/>
@@ -1126,11 +1128,11 @@
       <c r="C51" s="4" t="n"/>
       <c r="D51" s="2" t="n"/>
       <c r="E51" s="4" t="n"/>
-      <c r="F51" s="4" t="n"/>
+      <c r="F51" s="2" t="n"/>
       <c r="G51" s="2" t="n"/>
-      <c r="H51" s="2" t="n"/>
-      <c r="I51" s="5" t="n"/>
-      <c r="J51" s="6" t="n"/>
+      <c r="H51" s="5" t="n"/>
+      <c r="I51" s="6" t="n"/>
+      <c r="J51" s="7" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n"/>
@@ -1138,11 +1140,11 @@
       <c r="C52" s="4" t="n"/>
       <c r="D52" s="2" t="n"/>
       <c r="E52" s="4" t="n"/>
-      <c r="F52" s="4" t="n"/>
+      <c r="F52" s="2" t="n"/>
       <c r="G52" s="2" t="n"/>
-      <c r="H52" s="2" t="n"/>
-      <c r="I52" s="5" t="n"/>
-      <c r="J52" s="6" t="n"/>
+      <c r="H52" s="5" t="n"/>
+      <c r="I52" s="6" t="n"/>
+      <c r="J52" s="7" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n"/>
@@ -1150,11 +1152,11 @@
       <c r="C53" s="4" t="n"/>
       <c r="D53" s="2" t="n"/>
       <c r="E53" s="4" t="n"/>
-      <c r="F53" s="4" t="n"/>
+      <c r="F53" s="2" t="n"/>
       <c r="G53" s="2" t="n"/>
-      <c r="H53" s="2" t="n"/>
-      <c r="I53" s="5" t="n"/>
-      <c r="J53" s="6" t="n"/>
+      <c r="H53" s="5" t="n"/>
+      <c r="I53" s="6" t="n"/>
+      <c r="J53" s="7" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n"/>
@@ -1162,11 +1164,11 @@
       <c r="C54" s="4" t="n"/>
       <c r="D54" s="2" t="n"/>
       <c r="E54" s="4" t="n"/>
-      <c r="F54" s="4" t="n"/>
+      <c r="F54" s="2" t="n"/>
       <c r="G54" s="2" t="n"/>
-      <c r="H54" s="2" t="n"/>
-      <c r="I54" s="5" t="n"/>
-      <c r="J54" s="6" t="n"/>
+      <c r="H54" s="5" t="n"/>
+      <c r="I54" s="6" t="n"/>
+      <c r="J54" s="7" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n"/>
@@ -1174,11 +1176,11 @@
       <c r="C55" s="4" t="n"/>
       <c r="D55" s="2" t="n"/>
       <c r="E55" s="4" t="n"/>
-      <c r="F55" s="4" t="n"/>
+      <c r="F55" s="2" t="n"/>
       <c r="G55" s="2" t="n"/>
-      <c r="H55" s="2" t="n"/>
-      <c r="I55" s="5" t="n"/>
-      <c r="J55" s="6" t="n"/>
+      <c r="H55" s="5" t="n"/>
+      <c r="I55" s="6" t="n"/>
+      <c r="J55" s="7" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n"/>
@@ -1186,11 +1188,11 @@
       <c r="C56" s="4" t="n"/>
       <c r="D56" s="2" t="n"/>
       <c r="E56" s="4" t="n"/>
-      <c r="F56" s="4" t="n"/>
+      <c r="F56" s="2" t="n"/>
       <c r="G56" s="2" t="n"/>
-      <c r="H56" s="2" t="n"/>
-      <c r="I56" s="5" t="n"/>
-      <c r="J56" s="6" t="n"/>
+      <c r="H56" s="5" t="n"/>
+      <c r="I56" s="6" t="n"/>
+      <c r="J56" s="7" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n"/>
@@ -1198,11 +1200,11 @@
       <c r="C57" s="4" t="n"/>
       <c r="D57" s="2" t="n"/>
       <c r="E57" s="4" t="n"/>
-      <c r="F57" s="4" t="n"/>
+      <c r="F57" s="2" t="n"/>
       <c r="G57" s="2" t="n"/>
-      <c r="H57" s="2" t="n"/>
-      <c r="I57" s="5" t="n"/>
-      <c r="J57" s="6" t="n"/>
+      <c r="H57" s="5" t="n"/>
+      <c r="I57" s="6" t="n"/>
+      <c r="J57" s="7" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n"/>
@@ -1210,11 +1212,11 @@
       <c r="C58" s="4" t="n"/>
       <c r="D58" s="2" t="n"/>
       <c r="E58" s="4" t="n"/>
-      <c r="F58" s="4" t="n"/>
+      <c r="F58" s="2" t="n"/>
       <c r="G58" s="2" t="n"/>
-      <c r="H58" s="2" t="n"/>
-      <c r="I58" s="5" t="n"/>
-      <c r="J58" s="6" t="n"/>
+      <c r="H58" s="5" t="n"/>
+      <c r="I58" s="6" t="n"/>
+      <c r="J58" s="7" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n"/>
@@ -1222,11 +1224,11 @@
       <c r="C59" s="4" t="n"/>
       <c r="D59" s="2" t="n"/>
       <c r="E59" s="4" t="n"/>
-      <c r="F59" s="4" t="n"/>
+      <c r="F59" s="2" t="n"/>
       <c r="G59" s="2" t="n"/>
-      <c r="H59" s="2" t="n"/>
-      <c r="I59" s="5" t="n"/>
-      <c r="J59" s="6" t="n"/>
+      <c r="H59" s="5" t="n"/>
+      <c r="I59" s="6" t="n"/>
+      <c r="J59" s="7" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n"/>
@@ -1234,11 +1236,11 @@
       <c r="C60" s="4" t="n"/>
       <c r="D60" s="2" t="n"/>
       <c r="E60" s="4" t="n"/>
-      <c r="F60" s="4" t="n"/>
+      <c r="F60" s="2" t="n"/>
       <c r="G60" s="2" t="n"/>
-      <c r="H60" s="2" t="n"/>
-      <c r="I60" s="5" t="n"/>
-      <c r="J60" s="6" t="n"/>
+      <c r="H60" s="5" t="n"/>
+      <c r="I60" s="6" t="n"/>
+      <c r="J60" s="7" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n"/>
@@ -1246,11 +1248,11 @@
       <c r="C61" s="4" t="n"/>
       <c r="D61" s="2" t="n"/>
       <c r="E61" s="4" t="n"/>
-      <c r="F61" s="4" t="n"/>
+      <c r="F61" s="2" t="n"/>
       <c r="G61" s="2" t="n"/>
-      <c r="H61" s="2" t="n"/>
-      <c r="I61" s="5" t="n"/>
-      <c r="J61" s="6" t="n"/>
+      <c r="H61" s="5" t="n"/>
+      <c r="I61" s="6" t="n"/>
+      <c r="J61" s="7" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n"/>
@@ -1258,11 +1260,11 @@
       <c r="C62" s="4" t="n"/>
       <c r="D62" s="2" t="n"/>
       <c r="E62" s="4" t="n"/>
-      <c r="F62" s="4" t="n"/>
+      <c r="F62" s="2" t="n"/>
       <c r="G62" s="2" t="n"/>
-      <c r="H62" s="2" t="n"/>
-      <c r="I62" s="5" t="n"/>
-      <c r="J62" s="6" t="n"/>
+      <c r="H62" s="5" t="n"/>
+      <c r="I62" s="6" t="n"/>
+      <c r="J62" s="7" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n"/>
@@ -1270,11 +1272,11 @@
       <c r="C63" s="4" t="n"/>
       <c r="D63" s="2" t="n"/>
       <c r="E63" s="4" t="n"/>
-      <c r="F63" s="4" t="n"/>
+      <c r="F63" s="2" t="n"/>
       <c r="G63" s="2" t="n"/>
-      <c r="H63" s="2" t="n"/>
-      <c r="I63" s="5" t="n"/>
-      <c r="J63" s="6" t="n"/>
+      <c r="H63" s="5" t="n"/>
+      <c r="I63" s="6" t="n"/>
+      <c r="J63" s="7" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n"/>
@@ -1282,11 +1284,11 @@
       <c r="C64" s="4" t="n"/>
       <c r="D64" s="2" t="n"/>
       <c r="E64" s="4" t="n"/>
-      <c r="F64" s="4" t="n"/>
+      <c r="F64" s="2" t="n"/>
       <c r="G64" s="2" t="n"/>
-      <c r="H64" s="2" t="n"/>
-      <c r="I64" s="5" t="n"/>
-      <c r="J64" s="6" t="n"/>
+      <c r="H64" s="5" t="n"/>
+      <c r="I64" s="6" t="n"/>
+      <c r="J64" s="7" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n"/>
@@ -1294,11 +1296,11 @@
       <c r="C65" s="4" t="n"/>
       <c r="D65" s="2" t="n"/>
       <c r="E65" s="4" t="n"/>
-      <c r="F65" s="4" t="n"/>
+      <c r="F65" s="2" t="n"/>
       <c r="G65" s="2" t="n"/>
-      <c r="H65" s="2" t="n"/>
-      <c r="I65" s="5" t="n"/>
-      <c r="J65" s="6" t="n"/>
+      <c r="H65" s="5" t="n"/>
+      <c r="I65" s="6" t="n"/>
+      <c r="J65" s="7" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n"/>
@@ -1306,11 +1308,11 @@
       <c r="C66" s="4" t="n"/>
       <c r="D66" s="2" t="n"/>
       <c r="E66" s="4" t="n"/>
-      <c r="F66" s="4" t="n"/>
+      <c r="F66" s="2" t="n"/>
       <c r="G66" s="2" t="n"/>
-      <c r="H66" s="2" t="n"/>
-      <c r="I66" s="5" t="n"/>
-      <c r="J66" s="6" t="n"/>
+      <c r="H66" s="5" t="n"/>
+      <c r="I66" s="6" t="n"/>
+      <c r="J66" s="7" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n"/>
@@ -1318,11 +1320,11 @@
       <c r="C67" s="4" t="n"/>
       <c r="D67" s="2" t="n"/>
       <c r="E67" s="4" t="n"/>
-      <c r="F67" s="4" t="n"/>
+      <c r="F67" s="2" t="n"/>
       <c r="G67" s="2" t="n"/>
-      <c r="H67" s="2" t="n"/>
-      <c r="I67" s="5" t="n"/>
-      <c r="J67" s="6" t="n"/>
+      <c r="H67" s="5" t="n"/>
+      <c r="I67" s="6" t="n"/>
+      <c r="J67" s="7" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n"/>
@@ -1330,11 +1332,11 @@
       <c r="C68" s="4" t="n"/>
       <c r="D68" s="2" t="n"/>
       <c r="E68" s="4" t="n"/>
-      <c r="F68" s="4" t="n"/>
+      <c r="F68" s="2" t="n"/>
       <c r="G68" s="2" t="n"/>
-      <c r="H68" s="2" t="n"/>
-      <c r="I68" s="5" t="n"/>
-      <c r="J68" s="6" t="n"/>
+      <c r="H68" s="5" t="n"/>
+      <c r="I68" s="6" t="n"/>
+      <c r="J68" s="7" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n"/>
@@ -1342,11 +1344,11 @@
       <c r="C69" s="4" t="n"/>
       <c r="D69" s="2" t="n"/>
       <c r="E69" s="4" t="n"/>
-      <c r="F69" s="4" t="n"/>
+      <c r="F69" s="2" t="n"/>
       <c r="G69" s="2" t="n"/>
-      <c r="H69" s="2" t="n"/>
-      <c r="I69" s="5" t="n"/>
-      <c r="J69" s="6" t="n"/>
+      <c r="H69" s="5" t="n"/>
+      <c r="I69" s="6" t="n"/>
+      <c r="J69" s="7" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n"/>
@@ -1354,11 +1356,11 @@
       <c r="C70" s="4" t="n"/>
       <c r="D70" s="2" t="n"/>
       <c r="E70" s="4" t="n"/>
-      <c r="F70" s="4" t="n"/>
+      <c r="F70" s="2" t="n"/>
       <c r="G70" s="2" t="n"/>
-      <c r="H70" s="2" t="n"/>
-      <c r="I70" s="5" t="n"/>
-      <c r="J70" s="6" t="n"/>
+      <c r="H70" s="5" t="n"/>
+      <c r="I70" s="6" t="n"/>
+      <c r="J70" s="7" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n"/>
@@ -1366,11 +1368,11 @@
       <c r="C71" s="4" t="n"/>
       <c r="D71" s="2" t="n"/>
       <c r="E71" s="4" t="n"/>
-      <c r="F71" s="4" t="n"/>
+      <c r="F71" s="2" t="n"/>
       <c r="G71" s="2" t="n"/>
-      <c r="H71" s="2" t="n"/>
-      <c r="I71" s="5" t="n"/>
-      <c r="J71" s="6" t="n"/>
+      <c r="H71" s="5" t="n"/>
+      <c r="I71" s="6" t="n"/>
+      <c r="J71" s="7" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n"/>
@@ -1378,11 +1380,11 @@
       <c r="C72" s="4" t="n"/>
       <c r="D72" s="2" t="n"/>
       <c r="E72" s="4" t="n"/>
-      <c r="F72" s="4" t="n"/>
+      <c r="F72" s="2" t="n"/>
       <c r="G72" s="2" t="n"/>
-      <c r="H72" s="2" t="n"/>
-      <c r="I72" s="5" t="n"/>
-      <c r="J72" s="6" t="n"/>
+      <c r="H72" s="5" t="n"/>
+      <c r="I72" s="6" t="n"/>
+      <c r="J72" s="7" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n"/>
@@ -1390,11 +1392,11 @@
       <c r="C73" s="4" t="n"/>
       <c r="D73" s="2" t="n"/>
       <c r="E73" s="4" t="n"/>
-      <c r="F73" s="4" t="n"/>
+      <c r="F73" s="2" t="n"/>
       <c r="G73" s="2" t="n"/>
-      <c r="H73" s="2" t="n"/>
-      <c r="I73" s="5" t="n"/>
-      <c r="J73" s="6" t="n"/>
+      <c r="H73" s="5" t="n"/>
+      <c r="I73" s="6" t="n"/>
+      <c r="J73" s="7" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n"/>
@@ -1402,11 +1404,11 @@
       <c r="C74" s="4" t="n"/>
       <c r="D74" s="2" t="n"/>
       <c r="E74" s="4" t="n"/>
-      <c r="F74" s="4" t="n"/>
+      <c r="F74" s="2" t="n"/>
       <c r="G74" s="2" t="n"/>
-      <c r="H74" s="2" t="n"/>
-      <c r="I74" s="5" t="n"/>
-      <c r="J74" s="6" t="n"/>
+      <c r="H74" s="5" t="n"/>
+      <c r="I74" s="6" t="n"/>
+      <c r="J74" s="7" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n"/>
@@ -1414,11 +1416,11 @@
       <c r="C75" s="4" t="n"/>
       <c r="D75" s="2" t="n"/>
       <c r="E75" s="4" t="n"/>
-      <c r="F75" s="4" t="n"/>
+      <c r="F75" s="2" t="n"/>
       <c r="G75" s="2" t="n"/>
-      <c r="H75" s="2" t="n"/>
-      <c r="I75" s="5" t="n"/>
-      <c r="J75" s="6" t="n"/>
+      <c r="H75" s="5" t="n"/>
+      <c r="I75" s="6" t="n"/>
+      <c r="J75" s="7" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n"/>
@@ -1426,11 +1428,11 @@
       <c r="C76" s="4" t="n"/>
       <c r="D76" s="2" t="n"/>
       <c r="E76" s="4" t="n"/>
-      <c r="F76" s="4" t="n"/>
+      <c r="F76" s="2" t="n"/>
       <c r="G76" s="2" t="n"/>
-      <c r="H76" s="2" t="n"/>
-      <c r="I76" s="5" t="n"/>
-      <c r="J76" s="6" t="n"/>
+      <c r="H76" s="5" t="n"/>
+      <c r="I76" s="6" t="n"/>
+      <c r="J76" s="7" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n"/>
@@ -1438,11 +1440,11 @@
       <c r="C77" s="4" t="n"/>
       <c r="D77" s="2" t="n"/>
       <c r="E77" s="4" t="n"/>
-      <c r="F77" s="4" t="n"/>
+      <c r="F77" s="2" t="n"/>
       <c r="G77" s="2" t="n"/>
-      <c r="H77" s="2" t="n"/>
-      <c r="I77" s="5" t="n"/>
-      <c r="J77" s="6" t="n"/>
+      <c r="H77" s="5" t="n"/>
+      <c r="I77" s="6" t="n"/>
+      <c r="J77" s="7" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n"/>
@@ -1450,11 +1452,11 @@
       <c r="C78" s="4" t="n"/>
       <c r="D78" s="2" t="n"/>
       <c r="E78" s="4" t="n"/>
-      <c r="F78" s="4" t="n"/>
+      <c r="F78" s="2" t="n"/>
       <c r="G78" s="2" t="n"/>
-      <c r="H78" s="2" t="n"/>
-      <c r="I78" s="5" t="n"/>
-      <c r="J78" s="6" t="n"/>
+      <c r="H78" s="5" t="n"/>
+      <c r="I78" s="6" t="n"/>
+      <c r="J78" s="7" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n"/>
@@ -1462,11 +1464,11 @@
       <c r="C79" s="4" t="n"/>
       <c r="D79" s="2" t="n"/>
       <c r="E79" s="4" t="n"/>
-      <c r="F79" s="4" t="n"/>
+      <c r="F79" s="2" t="n"/>
       <c r="G79" s="2" t="n"/>
-      <c r="H79" s="2" t="n"/>
-      <c r="I79" s="5" t="n"/>
-      <c r="J79" s="6" t="n"/>
+      <c r="H79" s="5" t="n"/>
+      <c r="I79" s="6" t="n"/>
+      <c r="J79" s="7" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n"/>
@@ -1474,11 +1476,11 @@
       <c r="C80" s="4" t="n"/>
       <c r="D80" s="2" t="n"/>
       <c r="E80" s="4" t="n"/>
-      <c r="F80" s="4" t="n"/>
+      <c r="F80" s="2" t="n"/>
       <c r="G80" s="2" t="n"/>
-      <c r="H80" s="2" t="n"/>
-      <c r="I80" s="5" t="n"/>
-      <c r="J80" s="6" t="n"/>
+      <c r="H80" s="5" t="n"/>
+      <c r="I80" s="6" t="n"/>
+      <c r="J80" s="7" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n"/>
@@ -1486,11 +1488,11 @@
       <c r="C81" s="4" t="n"/>
       <c r="D81" s="2" t="n"/>
       <c r="E81" s="4" t="n"/>
-      <c r="F81" s="4" t="n"/>
+      <c r="F81" s="2" t="n"/>
       <c r="G81" s="2" t="n"/>
-      <c r="H81" s="2" t="n"/>
-      <c r="I81" s="5" t="n"/>
-      <c r="J81" s="6" t="n"/>
+      <c r="H81" s="5" t="n"/>
+      <c r="I81" s="6" t="n"/>
+      <c r="J81" s="7" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n"/>
@@ -1498,11 +1500,11 @@
       <c r="C82" s="4" t="n"/>
       <c r="D82" s="2" t="n"/>
       <c r="E82" s="4" t="n"/>
-      <c r="F82" s="4" t="n"/>
+      <c r="F82" s="2" t="n"/>
       <c r="G82" s="2" t="n"/>
-      <c r="H82" s="2" t="n"/>
-      <c r="I82" s="5" t="n"/>
-      <c r="J82" s="6" t="n"/>
+      <c r="H82" s="5" t="n"/>
+      <c r="I82" s="6" t="n"/>
+      <c r="J82" s="7" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n"/>
@@ -1510,11 +1512,11 @@
       <c r="C83" s="4" t="n"/>
       <c r="D83" s="2" t="n"/>
       <c r="E83" s="4" t="n"/>
-      <c r="F83" s="4" t="n"/>
+      <c r="F83" s="2" t="n"/>
       <c r="G83" s="2" t="n"/>
-      <c r="H83" s="2" t="n"/>
-      <c r="I83" s="5" t="n"/>
-      <c r="J83" s="6" t="n"/>
+      <c r="H83" s="5" t="n"/>
+      <c r="I83" s="6" t="n"/>
+      <c r="J83" s="7" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n"/>
@@ -1522,11 +1524,11 @@
       <c r="C84" s="4" t="n"/>
       <c r="D84" s="2" t="n"/>
       <c r="E84" s="4" t="n"/>
-      <c r="F84" s="4" t="n"/>
+      <c r="F84" s="2" t="n"/>
       <c r="G84" s="2" t="n"/>
-      <c r="H84" s="2" t="n"/>
-      <c r="I84" s="5" t="n"/>
-      <c r="J84" s="6" t="n"/>
+      <c r="H84" s="5" t="n"/>
+      <c r="I84" s="6" t="n"/>
+      <c r="J84" s="7" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n"/>
@@ -1534,11 +1536,11 @@
       <c r="C85" s="4" t="n"/>
       <c r="D85" s="2" t="n"/>
       <c r="E85" s="4" t="n"/>
-      <c r="F85" s="4" t="n"/>
+      <c r="F85" s="2" t="n"/>
       <c r="G85" s="2" t="n"/>
-      <c r="H85" s="2" t="n"/>
-      <c r="I85" s="5" t="n"/>
-      <c r="J85" s="6" t="n"/>
+      <c r="H85" s="5" t="n"/>
+      <c r="I85" s="6" t="n"/>
+      <c r="J85" s="7" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n"/>
@@ -1546,11 +1548,11 @@
       <c r="C86" s="4" t="n"/>
       <c r="D86" s="2" t="n"/>
       <c r="E86" s="4" t="n"/>
-      <c r="F86" s="4" t="n"/>
+      <c r="F86" s="2" t="n"/>
       <c r="G86" s="2" t="n"/>
-      <c r="H86" s="2" t="n"/>
-      <c r="I86" s="5" t="n"/>
-      <c r="J86" s="6" t="n"/>
+      <c r="H86" s="5" t="n"/>
+      <c r="I86" s="6" t="n"/>
+      <c r="J86" s="7" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n"/>
@@ -1558,11 +1560,11 @@
       <c r="C87" s="4" t="n"/>
       <c r="D87" s="2" t="n"/>
       <c r="E87" s="4" t="n"/>
-      <c r="F87" s="4" t="n"/>
+      <c r="F87" s="2" t="n"/>
       <c r="G87" s="2" t="n"/>
-      <c r="H87" s="2" t="n"/>
-      <c r="I87" s="5" t="n"/>
-      <c r="J87" s="6" t="n"/>
+      <c r="H87" s="5" t="n"/>
+      <c r="I87" s="6" t="n"/>
+      <c r="J87" s="7" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n"/>
@@ -1570,11 +1572,11 @@
       <c r="C88" s="4" t="n"/>
       <c r="D88" s="2" t="n"/>
       <c r="E88" s="4" t="n"/>
-      <c r="F88" s="4" t="n"/>
+      <c r="F88" s="2" t="n"/>
       <c r="G88" s="2" t="n"/>
-      <c r="H88" s="2" t="n"/>
-      <c r="I88" s="5" t="n"/>
-      <c r="J88" s="6" t="n"/>
+      <c r="H88" s="5" t="n"/>
+      <c r="I88" s="6" t="n"/>
+      <c r="J88" s="7" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n"/>
@@ -1582,11 +1584,11 @@
       <c r="C89" s="4" t="n"/>
       <c r="D89" s="2" t="n"/>
       <c r="E89" s="4" t="n"/>
-      <c r="F89" s="4" t="n"/>
+      <c r="F89" s="2" t="n"/>
       <c r="G89" s="2" t="n"/>
-      <c r="H89" s="2" t="n"/>
-      <c r="I89" s="5" t="n"/>
-      <c r="J89" s="6" t="n"/>
+      <c r="H89" s="5" t="n"/>
+      <c r="I89" s="6" t="n"/>
+      <c r="J89" s="7" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n"/>
@@ -1594,11 +1596,11 @@
       <c r="C90" s="4" t="n"/>
       <c r="D90" s="2" t="n"/>
       <c r="E90" s="4" t="n"/>
-      <c r="F90" s="4" t="n"/>
+      <c r="F90" s="2" t="n"/>
       <c r="G90" s="2" t="n"/>
-      <c r="H90" s="2" t="n"/>
-      <c r="I90" s="5" t="n"/>
-      <c r="J90" s="6" t="n"/>
+      <c r="H90" s="5" t="n"/>
+      <c r="I90" s="6" t="n"/>
+      <c r="J90" s="7" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n"/>
@@ -1606,11 +1608,11 @@
       <c r="C91" s="4" t="n"/>
       <c r="D91" s="2" t="n"/>
       <c r="E91" s="4" t="n"/>
-      <c r="F91" s="4" t="n"/>
+      <c r="F91" s="2" t="n"/>
       <c r="G91" s="2" t="n"/>
-      <c r="H91" s="2" t="n"/>
-      <c r="I91" s="5" t="n"/>
-      <c r="J91" s="6" t="n"/>
+      <c r="H91" s="5" t="n"/>
+      <c r="I91" s="6" t="n"/>
+      <c r="J91" s="7" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n"/>
@@ -1618,11 +1620,11 @@
       <c r="C92" s="4" t="n"/>
       <c r="D92" s="2" t="n"/>
       <c r="E92" s="4" t="n"/>
-      <c r="F92" s="4" t="n"/>
+      <c r="F92" s="2" t="n"/>
       <c r="G92" s="2" t="n"/>
-      <c r="H92" s="2" t="n"/>
-      <c r="I92" s="5" t="n"/>
-      <c r="J92" s="6" t="n"/>
+      <c r="H92" s="5" t="n"/>
+      <c r="I92" s="6" t="n"/>
+      <c r="J92" s="7" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n"/>
@@ -1630,11 +1632,11 @@
       <c r="C93" s="4" t="n"/>
       <c r="D93" s="2" t="n"/>
       <c r="E93" s="4" t="n"/>
-      <c r="F93" s="4" t="n"/>
+      <c r="F93" s="2" t="n"/>
       <c r="G93" s="2" t="n"/>
-      <c r="H93" s="2" t="n"/>
-      <c r="I93" s="5" t="n"/>
-      <c r="J93" s="6" t="n"/>
+      <c r="H93" s="5" t="n"/>
+      <c r="I93" s="6" t="n"/>
+      <c r="J93" s="7" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n"/>
@@ -1642,11 +1644,11 @@
       <c r="C94" s="4" t="n"/>
       <c r="D94" s="2" t="n"/>
       <c r="E94" s="4" t="n"/>
-      <c r="F94" s="4" t="n"/>
+      <c r="F94" s="2" t="n"/>
       <c r="G94" s="2" t="n"/>
-      <c r="H94" s="2" t="n"/>
-      <c r="I94" s="5" t="n"/>
-      <c r="J94" s="6" t="n"/>
+      <c r="H94" s="5" t="n"/>
+      <c r="I94" s="6" t="n"/>
+      <c r="J94" s="7" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n"/>
@@ -1654,11 +1656,11 @@
       <c r="C95" s="4" t="n"/>
       <c r="D95" s="2" t="n"/>
       <c r="E95" s="4" t="n"/>
-      <c r="F95" s="4" t="n"/>
+      <c r="F95" s="2" t="n"/>
       <c r="G95" s="2" t="n"/>
-      <c r="H95" s="2" t="n"/>
-      <c r="I95" s="5" t="n"/>
-      <c r="J95" s="6" t="n"/>
+      <c r="H95" s="5" t="n"/>
+      <c r="I95" s="6" t="n"/>
+      <c r="J95" s="7" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n"/>
@@ -1666,11 +1668,11 @@
       <c r="C96" s="4" t="n"/>
       <c r="D96" s="2" t="n"/>
       <c r="E96" s="4" t="n"/>
-      <c r="F96" s="4" t="n"/>
+      <c r="F96" s="2" t="n"/>
       <c r="G96" s="2" t="n"/>
-      <c r="H96" s="2" t="n"/>
-      <c r="I96" s="5" t="n"/>
-      <c r="J96" s="6" t="n"/>
+      <c r="H96" s="5" t="n"/>
+      <c r="I96" s="6" t="n"/>
+      <c r="J96" s="7" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n"/>
@@ -1678,11 +1680,11 @@
       <c r="C97" s="4" t="n"/>
       <c r="D97" s="2" t="n"/>
       <c r="E97" s="4" t="n"/>
-      <c r="F97" s="4" t="n"/>
+      <c r="F97" s="2" t="n"/>
       <c r="G97" s="2" t="n"/>
-      <c r="H97" s="2" t="n"/>
-      <c r="I97" s="5" t="n"/>
-      <c r="J97" s="6" t="n"/>
+      <c r="H97" s="5" t="n"/>
+      <c r="I97" s="6" t="n"/>
+      <c r="J97" s="7" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n"/>
@@ -1690,11 +1692,11 @@
       <c r="C98" s="4" t="n"/>
       <c r="D98" s="2" t="n"/>
       <c r="E98" s="4" t="n"/>
-      <c r="F98" s="4" t="n"/>
+      <c r="F98" s="2" t="n"/>
       <c r="G98" s="2" t="n"/>
-      <c r="H98" s="2" t="n"/>
-      <c r="I98" s="5" t="n"/>
-      <c r="J98" s="6" t="n"/>
+      <c r="H98" s="5" t="n"/>
+      <c r="I98" s="6" t="n"/>
+      <c r="J98" s="7" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n"/>
@@ -1702,11 +1704,11 @@
       <c r="C99" s="4" t="n"/>
       <c r="D99" s="2" t="n"/>
       <c r="E99" s="4" t="n"/>
-      <c r="F99" s="4" t="n"/>
+      <c r="F99" s="2" t="n"/>
       <c r="G99" s="2" t="n"/>
-      <c r="H99" s="2" t="n"/>
-      <c r="I99" s="5" t="n"/>
-      <c r="J99" s="6" t="n"/>
+      <c r="H99" s="5" t="n"/>
+      <c r="I99" s="6" t="n"/>
+      <c r="J99" s="7" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n"/>
@@ -1714,11 +1716,11 @@
       <c r="C100" s="4" t="n"/>
       <c r="D100" s="2" t="n"/>
       <c r="E100" s="4" t="n"/>
-      <c r="F100" s="4" t="n"/>
+      <c r="F100" s="2" t="n"/>
       <c r="G100" s="2" t="n"/>
-      <c r="H100" s="2" t="n"/>
-      <c r="I100" s="5" t="n"/>
-      <c r="J100" s="6" t="n"/>
+      <c r="H100" s="5" t="n"/>
+      <c r="I100" s="6" t="n"/>
+      <c r="J100" s="7" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n"/>
@@ -1726,11 +1728,11 @@
       <c r="C101" s="4" t="n"/>
       <c r="D101" s="2" t="n"/>
       <c r="E101" s="4" t="n"/>
-      <c r="F101" s="4" t="n"/>
+      <c r="F101" s="2" t="n"/>
       <c r="G101" s="2" t="n"/>
-      <c r="H101" s="2" t="n"/>
-      <c r="I101" s="5" t="n"/>
-      <c r="J101" s="6" t="n"/>
+      <c r="H101" s="5" t="n"/>
+      <c r="I101" s="6" t="n"/>
+      <c r="J101" s="7" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J101"/>
@@ -1739,15 +1741,12 @@
       <formula>AND($A2&lt;&gt;"",B2="")</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="3">
-    <dataValidation sqref="G2:G101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="2">
+    <dataValidation sqref="F2:F101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Kadın,Erkek"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Gerekmiyor,Başvuru yapılmadı,Başvuru yapıldı,Onaylandı,Reddedildi"</formula1>
-    </dataValidation>
-    <dataValidation sqref="F2:F101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="TCKN 11 haneli olmalıdır" type="textLength" operator="equal">
-      <formula1>11</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Widen availability column, add ROTA column
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F2bKD8QwZtMnPmjESyq7MM
</commit_message>
<xml_diff>
--- a/DiscoverEU_KA155_Katilimci_Tablosu.xlsx
+++ b/DiscoverEU_KA155_Katilimci_Tablosu.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tablo1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tablo1'!$A$1:$J$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tablo1'!$A$1:$K$101</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -79,19 +79,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -467,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J101"/>
+  <dimension ref="A1:K101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -478,8 +485,9 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="32" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -533,8 +541,13 @@
           <t>SEYAHAT TARİHLERİ</t>
         </is>
       </c>
-    </row>
-    <row r="2">
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>ROTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="n"/>
       <c r="B2" s="3" t="n"/>
       <c r="C2" s="4" t="n"/>
@@ -543,10 +556,11 @@
       <c r="F2" s="2" t="n"/>
       <c r="G2" s="2" t="n"/>
       <c r="H2" s="5" t="n"/>
-      <c r="I2" s="6" t="n"/>
-      <c r="J2" s="7" t="n"/>
-    </row>
-    <row r="3">
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="6" t="n"/>
+      <c r="K2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="32" customHeight="1">
       <c r="A3" s="2" t="n"/>
       <c r="B3" s="3" t="n"/>
       <c r="C3" s="4" t="n"/>
@@ -555,10 +569,11 @@
       <c r="F3" s="2" t="n"/>
       <c r="G3" s="2" t="n"/>
       <c r="H3" s="5" t="n"/>
-      <c r="I3" s="6" t="n"/>
-      <c r="J3" s="7" t="n"/>
-    </row>
-    <row r="4">
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="6" t="n"/>
+      <c r="K3" s="2" t="n"/>
+    </row>
+    <row r="4" ht="32" customHeight="1">
       <c r="A4" s="2" t="n"/>
       <c r="B4" s="3" t="n"/>
       <c r="C4" s="4" t="n"/>
@@ -567,10 +582,11 @@
       <c r="F4" s="2" t="n"/>
       <c r="G4" s="2" t="n"/>
       <c r="H4" s="5" t="n"/>
-      <c r="I4" s="6" t="n"/>
-      <c r="J4" s="7" t="n"/>
-    </row>
-    <row r="5">
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="6" t="n"/>
+      <c r="K4" s="2" t="n"/>
+    </row>
+    <row r="5" ht="32" customHeight="1">
       <c r="A5" s="2" t="n"/>
       <c r="B5" s="3" t="n"/>
       <c r="C5" s="4" t="n"/>
@@ -579,10 +595,11 @@
       <c r="F5" s="2" t="n"/>
       <c r="G5" s="2" t="n"/>
       <c r="H5" s="5" t="n"/>
-      <c r="I5" s="6" t="n"/>
-      <c r="J5" s="7" t="n"/>
-    </row>
-    <row r="6">
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="6" t="n"/>
+      <c r="K5" s="2" t="n"/>
+    </row>
+    <row r="6" ht="32" customHeight="1">
       <c r="A6" s="2" t="n"/>
       <c r="B6" s="3" t="n"/>
       <c r="C6" s="4" t="n"/>
@@ -591,10 +608,11 @@
       <c r="F6" s="2" t="n"/>
       <c r="G6" s="2" t="n"/>
       <c r="H6" s="5" t="n"/>
-      <c r="I6" s="6" t="n"/>
-      <c r="J6" s="7" t="n"/>
-    </row>
-    <row r="7">
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="6" t="n"/>
+      <c r="K6" s="2" t="n"/>
+    </row>
+    <row r="7" ht="32" customHeight="1">
       <c r="A7" s="2" t="n"/>
       <c r="B7" s="3" t="n"/>
       <c r="C7" s="4" t="n"/>
@@ -603,10 +621,11 @@
       <c r="F7" s="2" t="n"/>
       <c r="G7" s="2" t="n"/>
       <c r="H7" s="5" t="n"/>
-      <c r="I7" s="6" t="n"/>
-      <c r="J7" s="7" t="n"/>
-    </row>
-    <row r="8">
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="6" t="n"/>
+      <c r="K7" s="2" t="n"/>
+    </row>
+    <row r="8" ht="32" customHeight="1">
       <c r="A8" s="2" t="n"/>
       <c r="B8" s="3" t="n"/>
       <c r="C8" s="4" t="n"/>
@@ -615,10 +634,11 @@
       <c r="F8" s="2" t="n"/>
       <c r="G8" s="2" t="n"/>
       <c r="H8" s="5" t="n"/>
-      <c r="I8" s="6" t="n"/>
-      <c r="J8" s="7" t="n"/>
-    </row>
-    <row r="9">
+      <c r="I8" s="2" t="n"/>
+      <c r="J8" s="6" t="n"/>
+      <c r="K8" s="2" t="n"/>
+    </row>
+    <row r="9" ht="32" customHeight="1">
       <c r="A9" s="2" t="n"/>
       <c r="B9" s="3" t="n"/>
       <c r="C9" s="4" t="n"/>
@@ -627,10 +647,11 @@
       <c r="F9" s="2" t="n"/>
       <c r="G9" s="2" t="n"/>
       <c r="H9" s="5" t="n"/>
-      <c r="I9" s="6" t="n"/>
-      <c r="J9" s="7" t="n"/>
-    </row>
-    <row r="10">
+      <c r="I9" s="2" t="n"/>
+      <c r="J9" s="6" t="n"/>
+      <c r="K9" s="2" t="n"/>
+    </row>
+    <row r="10" ht="32" customHeight="1">
       <c r="A10" s="2" t="n"/>
       <c r="B10" s="3" t="n"/>
       <c r="C10" s="4" t="n"/>
@@ -639,10 +660,11 @@
       <c r="F10" s="2" t="n"/>
       <c r="G10" s="2" t="n"/>
       <c r="H10" s="5" t="n"/>
-      <c r="I10" s="6" t="n"/>
-      <c r="J10" s="7" t="n"/>
-    </row>
-    <row r="11">
+      <c r="I10" s="2" t="n"/>
+      <c r="J10" s="6" t="n"/>
+      <c r="K10" s="2" t="n"/>
+    </row>
+    <row r="11" ht="32" customHeight="1">
       <c r="A11" s="2" t="n"/>
       <c r="B11" s="3" t="n"/>
       <c r="C11" s="4" t="n"/>
@@ -651,10 +673,11 @@
       <c r="F11" s="2" t="n"/>
       <c r="G11" s="2" t="n"/>
       <c r="H11" s="5" t="n"/>
-      <c r="I11" s="6" t="n"/>
-      <c r="J11" s="7" t="n"/>
-    </row>
-    <row r="12">
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="6" t="n"/>
+      <c r="K11" s="2" t="n"/>
+    </row>
+    <row r="12" ht="32" customHeight="1">
       <c r="A12" s="2" t="n"/>
       <c r="B12" s="3" t="n"/>
       <c r="C12" s="4" t="n"/>
@@ -663,10 +686,11 @@
       <c r="F12" s="2" t="n"/>
       <c r="G12" s="2" t="n"/>
       <c r="H12" s="5" t="n"/>
-      <c r="I12" s="6" t="n"/>
-      <c r="J12" s="7" t="n"/>
-    </row>
-    <row r="13">
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" s="6" t="n"/>
+      <c r="K12" s="2" t="n"/>
+    </row>
+    <row r="13" ht="32" customHeight="1">
       <c r="A13" s="2" t="n"/>
       <c r="B13" s="3" t="n"/>
       <c r="C13" s="4" t="n"/>
@@ -675,10 +699,11 @@
       <c r="F13" s="2" t="n"/>
       <c r="G13" s="2" t="n"/>
       <c r="H13" s="5" t="n"/>
-      <c r="I13" s="6" t="n"/>
-      <c r="J13" s="7" t="n"/>
-    </row>
-    <row r="14">
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="6" t="n"/>
+      <c r="K13" s="2" t="n"/>
+    </row>
+    <row r="14" ht="32" customHeight="1">
       <c r="A14" s="2" t="n"/>
       <c r="B14" s="3" t="n"/>
       <c r="C14" s="4" t="n"/>
@@ -687,10 +712,11 @@
       <c r="F14" s="2" t="n"/>
       <c r="G14" s="2" t="n"/>
       <c r="H14" s="5" t="n"/>
-      <c r="I14" s="6" t="n"/>
-      <c r="J14" s="7" t="n"/>
-    </row>
-    <row r="15">
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="6" t="n"/>
+      <c r="K14" s="2" t="n"/>
+    </row>
+    <row r="15" ht="32" customHeight="1">
       <c r="A15" s="2" t="n"/>
       <c r="B15" s="3" t="n"/>
       <c r="C15" s="4" t="n"/>
@@ -699,10 +725,11 @@
       <c r="F15" s="2" t="n"/>
       <c r="G15" s="2" t="n"/>
       <c r="H15" s="5" t="n"/>
-      <c r="I15" s="6" t="n"/>
-      <c r="J15" s="7" t="n"/>
-    </row>
-    <row r="16">
+      <c r="I15" s="2" t="n"/>
+      <c r="J15" s="6" t="n"/>
+      <c r="K15" s="2" t="n"/>
+    </row>
+    <row r="16" ht="32" customHeight="1">
       <c r="A16" s="2" t="n"/>
       <c r="B16" s="3" t="n"/>
       <c r="C16" s="4" t="n"/>
@@ -711,10 +738,11 @@
       <c r="F16" s="2" t="n"/>
       <c r="G16" s="2" t="n"/>
       <c r="H16" s="5" t="n"/>
-      <c r="I16" s="6" t="n"/>
-      <c r="J16" s="7" t="n"/>
-    </row>
-    <row r="17">
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="6" t="n"/>
+      <c r="K16" s="2" t="n"/>
+    </row>
+    <row r="17" ht="32" customHeight="1">
       <c r="A17" s="2" t="n"/>
       <c r="B17" s="3" t="n"/>
       <c r="C17" s="4" t="n"/>
@@ -723,10 +751,11 @@
       <c r="F17" s="2" t="n"/>
       <c r="G17" s="2" t="n"/>
       <c r="H17" s="5" t="n"/>
-      <c r="I17" s="6" t="n"/>
-      <c r="J17" s="7" t="n"/>
-    </row>
-    <row r="18">
+      <c r="I17" s="2" t="n"/>
+      <c r="J17" s="6" t="n"/>
+      <c r="K17" s="2" t="n"/>
+    </row>
+    <row r="18" ht="32" customHeight="1">
       <c r="A18" s="2" t="n"/>
       <c r="B18" s="3" t="n"/>
       <c r="C18" s="4" t="n"/>
@@ -735,10 +764,11 @@
       <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="n"/>
       <c r="H18" s="5" t="n"/>
-      <c r="I18" s="6" t="n"/>
-      <c r="J18" s="7" t="n"/>
-    </row>
-    <row r="19">
+      <c r="I18" s="2" t="n"/>
+      <c r="J18" s="6" t="n"/>
+      <c r="K18" s="2" t="n"/>
+    </row>
+    <row r="19" ht="32" customHeight="1">
       <c r="A19" s="2" t="n"/>
       <c r="B19" s="3" t="n"/>
       <c r="C19" s="4" t="n"/>
@@ -747,10 +777,11 @@
       <c r="F19" s="2" t="n"/>
       <c r="G19" s="2" t="n"/>
       <c r="H19" s="5" t="n"/>
-      <c r="I19" s="6" t="n"/>
-      <c r="J19" s="7" t="n"/>
-    </row>
-    <row r="20">
+      <c r="I19" s="2" t="n"/>
+      <c r="J19" s="6" t="n"/>
+      <c r="K19" s="2" t="n"/>
+    </row>
+    <row r="20" ht="32" customHeight="1">
       <c r="A20" s="2" t="n"/>
       <c r="B20" s="3" t="n"/>
       <c r="C20" s="4" t="n"/>
@@ -759,10 +790,11 @@
       <c r="F20" s="2" t="n"/>
       <c r="G20" s="2" t="n"/>
       <c r="H20" s="5" t="n"/>
-      <c r="I20" s="6" t="n"/>
-      <c r="J20" s="7" t="n"/>
-    </row>
-    <row r="21">
+      <c r="I20" s="2" t="n"/>
+      <c r="J20" s="6" t="n"/>
+      <c r="K20" s="2" t="n"/>
+    </row>
+    <row r="21" ht="32" customHeight="1">
       <c r="A21" s="2" t="n"/>
       <c r="B21" s="3" t="n"/>
       <c r="C21" s="4" t="n"/>
@@ -771,10 +803,11 @@
       <c r="F21" s="2" t="n"/>
       <c r="G21" s="2" t="n"/>
       <c r="H21" s="5" t="n"/>
-      <c r="I21" s="6" t="n"/>
-      <c r="J21" s="7" t="n"/>
-    </row>
-    <row r="22">
+      <c r="I21" s="2" t="n"/>
+      <c r="J21" s="6" t="n"/>
+      <c r="K21" s="2" t="n"/>
+    </row>
+    <row r="22" ht="32" customHeight="1">
       <c r="A22" s="2" t="n"/>
       <c r="B22" s="3" t="n"/>
       <c r="C22" s="4" t="n"/>
@@ -783,10 +816,11 @@
       <c r="F22" s="2" t="n"/>
       <c r="G22" s="2" t="n"/>
       <c r="H22" s="5" t="n"/>
-      <c r="I22" s="6" t="n"/>
-      <c r="J22" s="7" t="n"/>
-    </row>
-    <row r="23">
+      <c r="I22" s="2" t="n"/>
+      <c r="J22" s="6" t="n"/>
+      <c r="K22" s="2" t="n"/>
+    </row>
+    <row r="23" ht="32" customHeight="1">
       <c r="A23" s="2" t="n"/>
       <c r="B23" s="3" t="n"/>
       <c r="C23" s="4" t="n"/>
@@ -795,10 +829,11 @@
       <c r="F23" s="2" t="n"/>
       <c r="G23" s="2" t="n"/>
       <c r="H23" s="5" t="n"/>
-      <c r="I23" s="6" t="n"/>
-      <c r="J23" s="7" t="n"/>
-    </row>
-    <row r="24">
+      <c r="I23" s="2" t="n"/>
+      <c r="J23" s="6" t="n"/>
+      <c r="K23" s="2" t="n"/>
+    </row>
+    <row r="24" ht="32" customHeight="1">
       <c r="A24" s="2" t="n"/>
       <c r="B24" s="3" t="n"/>
       <c r="C24" s="4" t="n"/>
@@ -807,10 +842,11 @@
       <c r="F24" s="2" t="n"/>
       <c r="G24" s="2" t="n"/>
       <c r="H24" s="5" t="n"/>
-      <c r="I24" s="6" t="n"/>
-      <c r="J24" s="7" t="n"/>
-    </row>
-    <row r="25">
+      <c r="I24" s="2" t="n"/>
+      <c r="J24" s="6" t="n"/>
+      <c r="K24" s="2" t="n"/>
+    </row>
+    <row r="25" ht="32" customHeight="1">
       <c r="A25" s="2" t="n"/>
       <c r="B25" s="3" t="n"/>
       <c r="C25" s="4" t="n"/>
@@ -819,10 +855,11 @@
       <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="n"/>
       <c r="H25" s="5" t="n"/>
-      <c r="I25" s="6" t="n"/>
-      <c r="J25" s="7" t="n"/>
-    </row>
-    <row r="26">
+      <c r="I25" s="2" t="n"/>
+      <c r="J25" s="6" t="n"/>
+      <c r="K25" s="2" t="n"/>
+    </row>
+    <row r="26" ht="32" customHeight="1">
       <c r="A26" s="2" t="n"/>
       <c r="B26" s="3" t="n"/>
       <c r="C26" s="4" t="n"/>
@@ -831,10 +868,11 @@
       <c r="F26" s="2" t="n"/>
       <c r="G26" s="2" t="n"/>
       <c r="H26" s="5" t="n"/>
-      <c r="I26" s="6" t="n"/>
-      <c r="J26" s="7" t="n"/>
-    </row>
-    <row r="27">
+      <c r="I26" s="2" t="n"/>
+      <c r="J26" s="6" t="n"/>
+      <c r="K26" s="2" t="n"/>
+    </row>
+    <row r="27" ht="32" customHeight="1">
       <c r="A27" s="2" t="n"/>
       <c r="B27" s="3" t="n"/>
       <c r="C27" s="4" t="n"/>
@@ -843,10 +881,11 @@
       <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="n"/>
       <c r="H27" s="5" t="n"/>
-      <c r="I27" s="6" t="n"/>
-      <c r="J27" s="7" t="n"/>
-    </row>
-    <row r="28">
+      <c r="I27" s="2" t="n"/>
+      <c r="J27" s="6" t="n"/>
+      <c r="K27" s="2" t="n"/>
+    </row>
+    <row r="28" ht="32" customHeight="1">
       <c r="A28" s="2" t="n"/>
       <c r="B28" s="3" t="n"/>
       <c r="C28" s="4" t="n"/>
@@ -855,10 +894,11 @@
       <c r="F28" s="2" t="n"/>
       <c r="G28" s="2" t="n"/>
       <c r="H28" s="5" t="n"/>
-      <c r="I28" s="6" t="n"/>
-      <c r="J28" s="7" t="n"/>
-    </row>
-    <row r="29">
+      <c r="I28" s="2" t="n"/>
+      <c r="J28" s="6" t="n"/>
+      <c r="K28" s="2" t="n"/>
+    </row>
+    <row r="29" ht="32" customHeight="1">
       <c r="A29" s="2" t="n"/>
       <c r="B29" s="3" t="n"/>
       <c r="C29" s="4" t="n"/>
@@ -867,10 +907,11 @@
       <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="n"/>
       <c r="H29" s="5" t="n"/>
-      <c r="I29" s="6" t="n"/>
-      <c r="J29" s="7" t="n"/>
-    </row>
-    <row r="30">
+      <c r="I29" s="2" t="n"/>
+      <c r="J29" s="6" t="n"/>
+      <c r="K29" s="2" t="n"/>
+    </row>
+    <row r="30" ht="32" customHeight="1">
       <c r="A30" s="2" t="n"/>
       <c r="B30" s="3" t="n"/>
       <c r="C30" s="4" t="n"/>
@@ -879,10 +920,11 @@
       <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="n"/>
       <c r="H30" s="5" t="n"/>
-      <c r="I30" s="6" t="n"/>
-      <c r="J30" s="7" t="n"/>
-    </row>
-    <row r="31">
+      <c r="I30" s="2" t="n"/>
+      <c r="J30" s="6" t="n"/>
+      <c r="K30" s="2" t="n"/>
+    </row>
+    <row r="31" ht="32" customHeight="1">
       <c r="A31" s="2" t="n"/>
       <c r="B31" s="3" t="n"/>
       <c r="C31" s="4" t="n"/>
@@ -891,10 +933,11 @@
       <c r="F31" s="2" t="n"/>
       <c r="G31" s="2" t="n"/>
       <c r="H31" s="5" t="n"/>
-      <c r="I31" s="6" t="n"/>
-      <c r="J31" s="7" t="n"/>
-    </row>
-    <row r="32">
+      <c r="I31" s="2" t="n"/>
+      <c r="J31" s="6" t="n"/>
+      <c r="K31" s="2" t="n"/>
+    </row>
+    <row r="32" ht="32" customHeight="1">
       <c r="A32" s="2" t="n"/>
       <c r="B32" s="3" t="n"/>
       <c r="C32" s="4" t="n"/>
@@ -903,10 +946,11 @@
       <c r="F32" s="2" t="n"/>
       <c r="G32" s="2" t="n"/>
       <c r="H32" s="5" t="n"/>
-      <c r="I32" s="6" t="n"/>
-      <c r="J32" s="7" t="n"/>
-    </row>
-    <row r="33">
+      <c r="I32" s="2" t="n"/>
+      <c r="J32" s="6" t="n"/>
+      <c r="K32" s="2" t="n"/>
+    </row>
+    <row r="33" ht="32" customHeight="1">
       <c r="A33" s="2" t="n"/>
       <c r="B33" s="3" t="n"/>
       <c r="C33" s="4" t="n"/>
@@ -915,10 +959,11 @@
       <c r="F33" s="2" t="n"/>
       <c r="G33" s="2" t="n"/>
       <c r="H33" s="5" t="n"/>
-      <c r="I33" s="6" t="n"/>
-      <c r="J33" s="7" t="n"/>
-    </row>
-    <row r="34">
+      <c r="I33" s="2" t="n"/>
+      <c r="J33" s="6" t="n"/>
+      <c r="K33" s="2" t="n"/>
+    </row>
+    <row r="34" ht="32" customHeight="1">
       <c r="A34" s="2" t="n"/>
       <c r="B34" s="3" t="n"/>
       <c r="C34" s="4" t="n"/>
@@ -927,10 +972,11 @@
       <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="n"/>
       <c r="H34" s="5" t="n"/>
-      <c r="I34" s="6" t="n"/>
-      <c r="J34" s="7" t="n"/>
-    </row>
-    <row r="35">
+      <c r="I34" s="2" t="n"/>
+      <c r="J34" s="6" t="n"/>
+      <c r="K34" s="2" t="n"/>
+    </row>
+    <row r="35" ht="32" customHeight="1">
       <c r="A35" s="2" t="n"/>
       <c r="B35" s="3" t="n"/>
       <c r="C35" s="4" t="n"/>
@@ -939,10 +985,11 @@
       <c r="F35" s="2" t="n"/>
       <c r="G35" s="2" t="n"/>
       <c r="H35" s="5" t="n"/>
-      <c r="I35" s="6" t="n"/>
-      <c r="J35" s="7" t="n"/>
-    </row>
-    <row r="36">
+      <c r="I35" s="2" t="n"/>
+      <c r="J35" s="6" t="n"/>
+      <c r="K35" s="2" t="n"/>
+    </row>
+    <row r="36" ht="32" customHeight="1">
       <c r="A36" s="2" t="n"/>
       <c r="B36" s="3" t="n"/>
       <c r="C36" s="4" t="n"/>
@@ -951,10 +998,11 @@
       <c r="F36" s="2" t="n"/>
       <c r="G36" s="2" t="n"/>
       <c r="H36" s="5" t="n"/>
-      <c r="I36" s="6" t="n"/>
-      <c r="J36" s="7" t="n"/>
-    </row>
-    <row r="37">
+      <c r="I36" s="2" t="n"/>
+      <c r="J36" s="6" t="n"/>
+      <c r="K36" s="2" t="n"/>
+    </row>
+    <row r="37" ht="32" customHeight="1">
       <c r="A37" s="2" t="n"/>
       <c r="B37" s="3" t="n"/>
       <c r="C37" s="4" t="n"/>
@@ -963,10 +1011,11 @@
       <c r="F37" s="2" t="n"/>
       <c r="G37" s="2" t="n"/>
       <c r="H37" s="5" t="n"/>
-      <c r="I37" s="6" t="n"/>
-      <c r="J37" s="7" t="n"/>
-    </row>
-    <row r="38">
+      <c r="I37" s="2" t="n"/>
+      <c r="J37" s="6" t="n"/>
+      <c r="K37" s="2" t="n"/>
+    </row>
+    <row r="38" ht="32" customHeight="1">
       <c r="A38" s="2" t="n"/>
       <c r="B38" s="3" t="n"/>
       <c r="C38" s="4" t="n"/>
@@ -975,10 +1024,11 @@
       <c r="F38" s="2" t="n"/>
       <c r="G38" s="2" t="n"/>
       <c r="H38" s="5" t="n"/>
-      <c r="I38" s="6" t="n"/>
-      <c r="J38" s="7" t="n"/>
-    </row>
-    <row r="39">
+      <c r="I38" s="2" t="n"/>
+      <c r="J38" s="6" t="n"/>
+      <c r="K38" s="2" t="n"/>
+    </row>
+    <row r="39" ht="32" customHeight="1">
       <c r="A39" s="2" t="n"/>
       <c r="B39" s="3" t="n"/>
       <c r="C39" s="4" t="n"/>
@@ -987,10 +1037,11 @@
       <c r="F39" s="2" t="n"/>
       <c r="G39" s="2" t="n"/>
       <c r="H39" s="5" t="n"/>
-      <c r="I39" s="6" t="n"/>
-      <c r="J39" s="7" t="n"/>
-    </row>
-    <row r="40">
+      <c r="I39" s="2" t="n"/>
+      <c r="J39" s="6" t="n"/>
+      <c r="K39" s="2" t="n"/>
+    </row>
+    <row r="40" ht="32" customHeight="1">
       <c r="A40" s="2" t="n"/>
       <c r="B40" s="3" t="n"/>
       <c r="C40" s="4" t="n"/>
@@ -999,10 +1050,11 @@
       <c r="F40" s="2" t="n"/>
       <c r="G40" s="2" t="n"/>
       <c r="H40" s="5" t="n"/>
-      <c r="I40" s="6" t="n"/>
-      <c r="J40" s="7" t="n"/>
-    </row>
-    <row r="41">
+      <c r="I40" s="2" t="n"/>
+      <c r="J40" s="6" t="n"/>
+      <c r="K40" s="2" t="n"/>
+    </row>
+    <row r="41" ht="32" customHeight="1">
       <c r="A41" s="2" t="n"/>
       <c r="B41" s="3" t="n"/>
       <c r="C41" s="4" t="n"/>
@@ -1011,10 +1063,11 @@
       <c r="F41" s="2" t="n"/>
       <c r="G41" s="2" t="n"/>
       <c r="H41" s="5" t="n"/>
-      <c r="I41" s="6" t="n"/>
-      <c r="J41" s="7" t="n"/>
-    </row>
-    <row r="42">
+      <c r="I41" s="2" t="n"/>
+      <c r="J41" s="6" t="n"/>
+      <c r="K41" s="2" t="n"/>
+    </row>
+    <row r="42" ht="32" customHeight="1">
       <c r="A42" s="2" t="n"/>
       <c r="B42" s="3" t="n"/>
       <c r="C42" s="4" t="n"/>
@@ -1023,10 +1076,11 @@
       <c r="F42" s="2" t="n"/>
       <c r="G42" s="2" t="n"/>
       <c r="H42" s="5" t="n"/>
-      <c r="I42" s="6" t="n"/>
-      <c r="J42" s="7" t="n"/>
-    </row>
-    <row r="43">
+      <c r="I42" s="2" t="n"/>
+      <c r="J42" s="6" t="n"/>
+      <c r="K42" s="2" t="n"/>
+    </row>
+    <row r="43" ht="32" customHeight="1">
       <c r="A43" s="2" t="n"/>
       <c r="B43" s="3" t="n"/>
       <c r="C43" s="4" t="n"/>
@@ -1035,10 +1089,11 @@
       <c r="F43" s="2" t="n"/>
       <c r="G43" s="2" t="n"/>
       <c r="H43" s="5" t="n"/>
-      <c r="I43" s="6" t="n"/>
-      <c r="J43" s="7" t="n"/>
-    </row>
-    <row r="44">
+      <c r="I43" s="2" t="n"/>
+      <c r="J43" s="6" t="n"/>
+      <c r="K43" s="2" t="n"/>
+    </row>
+    <row r="44" ht="32" customHeight="1">
       <c r="A44" s="2" t="n"/>
       <c r="B44" s="3" t="n"/>
       <c r="C44" s="4" t="n"/>
@@ -1047,10 +1102,11 @@
       <c r="F44" s="2" t="n"/>
       <c r="G44" s="2" t="n"/>
       <c r="H44" s="5" t="n"/>
-      <c r="I44" s="6" t="n"/>
-      <c r="J44" s="7" t="n"/>
-    </row>
-    <row r="45">
+      <c r="I44" s="2" t="n"/>
+      <c r="J44" s="6" t="n"/>
+      <c r="K44" s="2" t="n"/>
+    </row>
+    <row r="45" ht="32" customHeight="1">
       <c r="A45" s="2" t="n"/>
       <c r="B45" s="3" t="n"/>
       <c r="C45" s="4" t="n"/>
@@ -1059,10 +1115,11 @@
       <c r="F45" s="2" t="n"/>
       <c r="G45" s="2" t="n"/>
       <c r="H45" s="5" t="n"/>
-      <c r="I45" s="6" t="n"/>
-      <c r="J45" s="7" t="n"/>
-    </row>
-    <row r="46">
+      <c r="I45" s="2" t="n"/>
+      <c r="J45" s="6" t="n"/>
+      <c r="K45" s="2" t="n"/>
+    </row>
+    <row r="46" ht="32" customHeight="1">
       <c r="A46" s="2" t="n"/>
       <c r="B46" s="3" t="n"/>
       <c r="C46" s="4" t="n"/>
@@ -1071,10 +1128,11 @@
       <c r="F46" s="2" t="n"/>
       <c r="G46" s="2" t="n"/>
       <c r="H46" s="5" t="n"/>
-      <c r="I46" s="6" t="n"/>
-      <c r="J46" s="7" t="n"/>
-    </row>
-    <row r="47">
+      <c r="I46" s="2" t="n"/>
+      <c r="J46" s="6" t="n"/>
+      <c r="K46" s="2" t="n"/>
+    </row>
+    <row r="47" ht="32" customHeight="1">
       <c r="A47" s="2" t="n"/>
       <c r="B47" s="3" t="n"/>
       <c r="C47" s="4" t="n"/>
@@ -1083,10 +1141,11 @@
       <c r="F47" s="2" t="n"/>
       <c r="G47" s="2" t="n"/>
       <c r="H47" s="5" t="n"/>
-      <c r="I47" s="6" t="n"/>
-      <c r="J47" s="7" t="n"/>
-    </row>
-    <row r="48">
+      <c r="I47" s="2" t="n"/>
+      <c r="J47" s="6" t="n"/>
+      <c r="K47" s="2" t="n"/>
+    </row>
+    <row r="48" ht="32" customHeight="1">
       <c r="A48" s="2" t="n"/>
       <c r="B48" s="3" t="n"/>
       <c r="C48" s="4" t="n"/>
@@ -1095,10 +1154,11 @@
       <c r="F48" s="2" t="n"/>
       <c r="G48" s="2" t="n"/>
       <c r="H48" s="5" t="n"/>
-      <c r="I48" s="6" t="n"/>
-      <c r="J48" s="7" t="n"/>
-    </row>
-    <row r="49">
+      <c r="I48" s="2" t="n"/>
+      <c r="J48" s="6" t="n"/>
+      <c r="K48" s="2" t="n"/>
+    </row>
+    <row r="49" ht="32" customHeight="1">
       <c r="A49" s="2" t="n"/>
       <c r="B49" s="3" t="n"/>
       <c r="C49" s="4" t="n"/>
@@ -1107,10 +1167,11 @@
       <c r="F49" s="2" t="n"/>
       <c r="G49" s="2" t="n"/>
       <c r="H49" s="5" t="n"/>
-      <c r="I49" s="6" t="n"/>
-      <c r="J49" s="7" t="n"/>
-    </row>
-    <row r="50">
+      <c r="I49" s="2" t="n"/>
+      <c r="J49" s="6" t="n"/>
+      <c r="K49" s="2" t="n"/>
+    </row>
+    <row r="50" ht="32" customHeight="1">
       <c r="A50" s="2" t="n"/>
       <c r="B50" s="3" t="n"/>
       <c r="C50" s="4" t="n"/>
@@ -1119,10 +1180,11 @@
       <c r="F50" s="2" t="n"/>
       <c r="G50" s="2" t="n"/>
       <c r="H50" s="5" t="n"/>
-      <c r="I50" s="6" t="n"/>
-      <c r="J50" s="7" t="n"/>
-    </row>
-    <row r="51">
+      <c r="I50" s="2" t="n"/>
+      <c r="J50" s="6" t="n"/>
+      <c r="K50" s="2" t="n"/>
+    </row>
+    <row r="51" ht="32" customHeight="1">
       <c r="A51" s="2" t="n"/>
       <c r="B51" s="3" t="n"/>
       <c r="C51" s="4" t="n"/>
@@ -1131,10 +1193,11 @@
       <c r="F51" s="2" t="n"/>
       <c r="G51" s="2" t="n"/>
       <c r="H51" s="5" t="n"/>
-      <c r="I51" s="6" t="n"/>
-      <c r="J51" s="7" t="n"/>
-    </row>
-    <row r="52">
+      <c r="I51" s="2" t="n"/>
+      <c r="J51" s="6" t="n"/>
+      <c r="K51" s="2" t="n"/>
+    </row>
+    <row r="52" ht="32" customHeight="1">
       <c r="A52" s="2" t="n"/>
       <c r="B52" s="3" t="n"/>
       <c r="C52" s="4" t="n"/>
@@ -1143,10 +1206,11 @@
       <c r="F52" s="2" t="n"/>
       <c r="G52" s="2" t="n"/>
       <c r="H52" s="5" t="n"/>
-      <c r="I52" s="6" t="n"/>
-      <c r="J52" s="7" t="n"/>
-    </row>
-    <row r="53">
+      <c r="I52" s="2" t="n"/>
+      <c r="J52" s="6" t="n"/>
+      <c r="K52" s="2" t="n"/>
+    </row>
+    <row r="53" ht="32" customHeight="1">
       <c r="A53" s="2" t="n"/>
       <c r="B53" s="3" t="n"/>
       <c r="C53" s="4" t="n"/>
@@ -1155,10 +1219,11 @@
       <c r="F53" s="2" t="n"/>
       <c r="G53" s="2" t="n"/>
       <c r="H53" s="5" t="n"/>
-      <c r="I53" s="6" t="n"/>
-      <c r="J53" s="7" t="n"/>
-    </row>
-    <row r="54">
+      <c r="I53" s="2" t="n"/>
+      <c r="J53" s="6" t="n"/>
+      <c r="K53" s="2" t="n"/>
+    </row>
+    <row r="54" ht="32" customHeight="1">
       <c r="A54" s="2" t="n"/>
       <c r="B54" s="3" t="n"/>
       <c r="C54" s="4" t="n"/>
@@ -1167,10 +1232,11 @@
       <c r="F54" s="2" t="n"/>
       <c r="G54" s="2" t="n"/>
       <c r="H54" s="5" t="n"/>
-      <c r="I54" s="6" t="n"/>
-      <c r="J54" s="7" t="n"/>
-    </row>
-    <row r="55">
+      <c r="I54" s="2" t="n"/>
+      <c r="J54" s="6" t="n"/>
+      <c r="K54" s="2" t="n"/>
+    </row>
+    <row r="55" ht="32" customHeight="1">
       <c r="A55" s="2" t="n"/>
       <c r="B55" s="3" t="n"/>
       <c r="C55" s="4" t="n"/>
@@ -1179,10 +1245,11 @@
       <c r="F55" s="2" t="n"/>
       <c r="G55" s="2" t="n"/>
       <c r="H55" s="5" t="n"/>
-      <c r="I55" s="6" t="n"/>
-      <c r="J55" s="7" t="n"/>
-    </row>
-    <row r="56">
+      <c r="I55" s="2" t="n"/>
+      <c r="J55" s="6" t="n"/>
+      <c r="K55" s="2" t="n"/>
+    </row>
+    <row r="56" ht="32" customHeight="1">
       <c r="A56" s="2" t="n"/>
       <c r="B56" s="3" t="n"/>
       <c r="C56" s="4" t="n"/>
@@ -1191,10 +1258,11 @@
       <c r="F56" s="2" t="n"/>
       <c r="G56" s="2" t="n"/>
       <c r="H56" s="5" t="n"/>
-      <c r="I56" s="6" t="n"/>
-      <c r="J56" s="7" t="n"/>
-    </row>
-    <row r="57">
+      <c r="I56" s="2" t="n"/>
+      <c r="J56" s="6" t="n"/>
+      <c r="K56" s="2" t="n"/>
+    </row>
+    <row r="57" ht="32" customHeight="1">
       <c r="A57" s="2" t="n"/>
       <c r="B57" s="3" t="n"/>
       <c r="C57" s="4" t="n"/>
@@ -1203,10 +1271,11 @@
       <c r="F57" s="2" t="n"/>
       <c r="G57" s="2" t="n"/>
       <c r="H57" s="5" t="n"/>
-      <c r="I57" s="6" t="n"/>
-      <c r="J57" s="7" t="n"/>
-    </row>
-    <row r="58">
+      <c r="I57" s="2" t="n"/>
+      <c r="J57" s="6" t="n"/>
+      <c r="K57" s="2" t="n"/>
+    </row>
+    <row r="58" ht="32" customHeight="1">
       <c r="A58" s="2" t="n"/>
       <c r="B58" s="3" t="n"/>
       <c r="C58" s="4" t="n"/>
@@ -1215,10 +1284,11 @@
       <c r="F58" s="2" t="n"/>
       <c r="G58" s="2" t="n"/>
       <c r="H58" s="5" t="n"/>
-      <c r="I58" s="6" t="n"/>
-      <c r="J58" s="7" t="n"/>
-    </row>
-    <row r="59">
+      <c r="I58" s="2" t="n"/>
+      <c r="J58" s="6" t="n"/>
+      <c r="K58" s="2" t="n"/>
+    </row>
+    <row r="59" ht="32" customHeight="1">
       <c r="A59" s="2" t="n"/>
       <c r="B59" s="3" t="n"/>
       <c r="C59" s="4" t="n"/>
@@ -1227,10 +1297,11 @@
       <c r="F59" s="2" t="n"/>
       <c r="G59" s="2" t="n"/>
       <c r="H59" s="5" t="n"/>
-      <c r="I59" s="6" t="n"/>
-      <c r="J59" s="7" t="n"/>
-    </row>
-    <row r="60">
+      <c r="I59" s="2" t="n"/>
+      <c r="J59" s="6" t="n"/>
+      <c r="K59" s="2" t="n"/>
+    </row>
+    <row r="60" ht="32" customHeight="1">
       <c r="A60" s="2" t="n"/>
       <c r="B60" s="3" t="n"/>
       <c r="C60" s="4" t="n"/>
@@ -1239,10 +1310,11 @@
       <c r="F60" s="2" t="n"/>
       <c r="G60" s="2" t="n"/>
       <c r="H60" s="5" t="n"/>
-      <c r="I60" s="6" t="n"/>
-      <c r="J60" s="7" t="n"/>
-    </row>
-    <row r="61">
+      <c r="I60" s="2" t="n"/>
+      <c r="J60" s="6" t="n"/>
+      <c r="K60" s="2" t="n"/>
+    </row>
+    <row r="61" ht="32" customHeight="1">
       <c r="A61" s="2" t="n"/>
       <c r="B61" s="3" t="n"/>
       <c r="C61" s="4" t="n"/>
@@ -1251,10 +1323,11 @@
       <c r="F61" s="2" t="n"/>
       <c r="G61" s="2" t="n"/>
       <c r="H61" s="5" t="n"/>
-      <c r="I61" s="6" t="n"/>
-      <c r="J61" s="7" t="n"/>
-    </row>
-    <row r="62">
+      <c r="I61" s="2" t="n"/>
+      <c r="J61" s="6" t="n"/>
+      <c r="K61" s="2" t="n"/>
+    </row>
+    <row r="62" ht="32" customHeight="1">
       <c r="A62" s="2" t="n"/>
       <c r="B62" s="3" t="n"/>
       <c r="C62" s="4" t="n"/>
@@ -1263,10 +1336,11 @@
       <c r="F62" s="2" t="n"/>
       <c r="G62" s="2" t="n"/>
       <c r="H62" s="5" t="n"/>
-      <c r="I62" s="6" t="n"/>
-      <c r="J62" s="7" t="n"/>
-    </row>
-    <row r="63">
+      <c r="I62" s="2" t="n"/>
+      <c r="J62" s="6" t="n"/>
+      <c r="K62" s="2" t="n"/>
+    </row>
+    <row r="63" ht="32" customHeight="1">
       <c r="A63" s="2" t="n"/>
       <c r="B63" s="3" t="n"/>
       <c r="C63" s="4" t="n"/>
@@ -1275,10 +1349,11 @@
       <c r="F63" s="2" t="n"/>
       <c r="G63" s="2" t="n"/>
       <c r="H63" s="5" t="n"/>
-      <c r="I63" s="6" t="n"/>
-      <c r="J63" s="7" t="n"/>
-    </row>
-    <row r="64">
+      <c r="I63" s="2" t="n"/>
+      <c r="J63" s="6" t="n"/>
+      <c r="K63" s="2" t="n"/>
+    </row>
+    <row r="64" ht="32" customHeight="1">
       <c r="A64" s="2" t="n"/>
       <c r="B64" s="3" t="n"/>
       <c r="C64" s="4" t="n"/>
@@ -1287,10 +1362,11 @@
       <c r="F64" s="2" t="n"/>
       <c r="G64" s="2" t="n"/>
       <c r="H64" s="5" t="n"/>
-      <c r="I64" s="6" t="n"/>
-      <c r="J64" s="7" t="n"/>
-    </row>
-    <row r="65">
+      <c r="I64" s="2" t="n"/>
+      <c r="J64" s="6" t="n"/>
+      <c r="K64" s="2" t="n"/>
+    </row>
+    <row r="65" ht="32" customHeight="1">
       <c r="A65" s="2" t="n"/>
       <c r="B65" s="3" t="n"/>
       <c r="C65" s="4" t="n"/>
@@ -1299,10 +1375,11 @@
       <c r="F65" s="2" t="n"/>
       <c r="G65" s="2" t="n"/>
       <c r="H65" s="5" t="n"/>
-      <c r="I65" s="6" t="n"/>
-      <c r="J65" s="7" t="n"/>
-    </row>
-    <row r="66">
+      <c r="I65" s="2" t="n"/>
+      <c r="J65" s="6" t="n"/>
+      <c r="K65" s="2" t="n"/>
+    </row>
+    <row r="66" ht="32" customHeight="1">
       <c r="A66" s="2" t="n"/>
       <c r="B66" s="3" t="n"/>
       <c r="C66" s="4" t="n"/>
@@ -1311,10 +1388,11 @@
       <c r="F66" s="2" t="n"/>
       <c r="G66" s="2" t="n"/>
       <c r="H66" s="5" t="n"/>
-      <c r="I66" s="6" t="n"/>
-      <c r="J66" s="7" t="n"/>
-    </row>
-    <row r="67">
+      <c r="I66" s="2" t="n"/>
+      <c r="J66" s="6" t="n"/>
+      <c r="K66" s="2" t="n"/>
+    </row>
+    <row r="67" ht="32" customHeight="1">
       <c r="A67" s="2" t="n"/>
       <c r="B67" s="3" t="n"/>
       <c r="C67" s="4" t="n"/>
@@ -1323,10 +1401,11 @@
       <c r="F67" s="2" t="n"/>
       <c r="G67" s="2" t="n"/>
       <c r="H67" s="5" t="n"/>
-      <c r="I67" s="6" t="n"/>
-      <c r="J67" s="7" t="n"/>
-    </row>
-    <row r="68">
+      <c r="I67" s="2" t="n"/>
+      <c r="J67" s="6" t="n"/>
+      <c r="K67" s="2" t="n"/>
+    </row>
+    <row r="68" ht="32" customHeight="1">
       <c r="A68" s="2" t="n"/>
       <c r="B68" s="3" t="n"/>
       <c r="C68" s="4" t="n"/>
@@ -1335,10 +1414,11 @@
       <c r="F68" s="2" t="n"/>
       <c r="G68" s="2" t="n"/>
       <c r="H68" s="5" t="n"/>
-      <c r="I68" s="6" t="n"/>
-      <c r="J68" s="7" t="n"/>
-    </row>
-    <row r="69">
+      <c r="I68" s="2" t="n"/>
+      <c r="J68" s="6" t="n"/>
+      <c r="K68" s="2" t="n"/>
+    </row>
+    <row r="69" ht="32" customHeight="1">
       <c r="A69" s="2" t="n"/>
       <c r="B69" s="3" t="n"/>
       <c r="C69" s="4" t="n"/>
@@ -1347,10 +1427,11 @@
       <c r="F69" s="2" t="n"/>
       <c r="G69" s="2" t="n"/>
       <c r="H69" s="5" t="n"/>
-      <c r="I69" s="6" t="n"/>
-      <c r="J69" s="7" t="n"/>
-    </row>
-    <row r="70">
+      <c r="I69" s="2" t="n"/>
+      <c r="J69" s="6" t="n"/>
+      <c r="K69" s="2" t="n"/>
+    </row>
+    <row r="70" ht="32" customHeight="1">
       <c r="A70" s="2" t="n"/>
       <c r="B70" s="3" t="n"/>
       <c r="C70" s="4" t="n"/>
@@ -1359,10 +1440,11 @@
       <c r="F70" s="2" t="n"/>
       <c r="G70" s="2" t="n"/>
       <c r="H70" s="5" t="n"/>
-      <c r="I70" s="6" t="n"/>
-      <c r="J70" s="7" t="n"/>
-    </row>
-    <row r="71">
+      <c r="I70" s="2" t="n"/>
+      <c r="J70" s="6" t="n"/>
+      <c r="K70" s="2" t="n"/>
+    </row>
+    <row r="71" ht="32" customHeight="1">
       <c r="A71" s="2" t="n"/>
       <c r="B71" s="3" t="n"/>
       <c r="C71" s="4" t="n"/>
@@ -1371,10 +1453,11 @@
       <c r="F71" s="2" t="n"/>
       <c r="G71" s="2" t="n"/>
       <c r="H71" s="5" t="n"/>
-      <c r="I71" s="6" t="n"/>
-      <c r="J71" s="7" t="n"/>
-    </row>
-    <row r="72">
+      <c r="I71" s="2" t="n"/>
+      <c r="J71" s="6" t="n"/>
+      <c r="K71" s="2" t="n"/>
+    </row>
+    <row r="72" ht="32" customHeight="1">
       <c r="A72" s="2" t="n"/>
       <c r="B72" s="3" t="n"/>
       <c r="C72" s="4" t="n"/>
@@ -1383,10 +1466,11 @@
       <c r="F72" s="2" t="n"/>
       <c r="G72" s="2" t="n"/>
       <c r="H72" s="5" t="n"/>
-      <c r="I72" s="6" t="n"/>
-      <c r="J72" s="7" t="n"/>
-    </row>
-    <row r="73">
+      <c r="I72" s="2" t="n"/>
+      <c r="J72" s="6" t="n"/>
+      <c r="K72" s="2" t="n"/>
+    </row>
+    <row r="73" ht="32" customHeight="1">
       <c r="A73" s="2" t="n"/>
       <c r="B73" s="3" t="n"/>
       <c r="C73" s="4" t="n"/>
@@ -1395,10 +1479,11 @@
       <c r="F73" s="2" t="n"/>
       <c r="G73" s="2" t="n"/>
       <c r="H73" s="5" t="n"/>
-      <c r="I73" s="6" t="n"/>
-      <c r="J73" s="7" t="n"/>
-    </row>
-    <row r="74">
+      <c r="I73" s="2" t="n"/>
+      <c r="J73" s="6" t="n"/>
+      <c r="K73" s="2" t="n"/>
+    </row>
+    <row r="74" ht="32" customHeight="1">
       <c r="A74" s="2" t="n"/>
       <c r="B74" s="3" t="n"/>
       <c r="C74" s="4" t="n"/>
@@ -1407,10 +1492,11 @@
       <c r="F74" s="2" t="n"/>
       <c r="G74" s="2" t="n"/>
       <c r="H74" s="5" t="n"/>
-      <c r="I74" s="6" t="n"/>
-      <c r="J74" s="7" t="n"/>
-    </row>
-    <row r="75">
+      <c r="I74" s="2" t="n"/>
+      <c r="J74" s="6" t="n"/>
+      <c r="K74" s="2" t="n"/>
+    </row>
+    <row r="75" ht="32" customHeight="1">
       <c r="A75" s="2" t="n"/>
       <c r="B75" s="3" t="n"/>
       <c r="C75" s="4" t="n"/>
@@ -1419,10 +1505,11 @@
       <c r="F75" s="2" t="n"/>
       <c r="G75" s="2" t="n"/>
       <c r="H75" s="5" t="n"/>
-      <c r="I75" s="6" t="n"/>
-      <c r="J75" s="7" t="n"/>
-    </row>
-    <row r="76">
+      <c r="I75" s="2" t="n"/>
+      <c r="J75" s="6" t="n"/>
+      <c r="K75" s="2" t="n"/>
+    </row>
+    <row r="76" ht="32" customHeight="1">
       <c r="A76" s="2" t="n"/>
       <c r="B76" s="3" t="n"/>
       <c r="C76" s="4" t="n"/>
@@ -1431,10 +1518,11 @@
       <c r="F76" s="2" t="n"/>
       <c r="G76" s="2" t="n"/>
       <c r="H76" s="5" t="n"/>
-      <c r="I76" s="6" t="n"/>
-      <c r="J76" s="7" t="n"/>
-    </row>
-    <row r="77">
+      <c r="I76" s="2" t="n"/>
+      <c r="J76" s="6" t="n"/>
+      <c r="K76" s="2" t="n"/>
+    </row>
+    <row r="77" ht="32" customHeight="1">
       <c r="A77" s="2" t="n"/>
       <c r="B77" s="3" t="n"/>
       <c r="C77" s="4" t="n"/>
@@ -1443,10 +1531,11 @@
       <c r="F77" s="2" t="n"/>
       <c r="G77" s="2" t="n"/>
       <c r="H77" s="5" t="n"/>
-      <c r="I77" s="6" t="n"/>
-      <c r="J77" s="7" t="n"/>
-    </row>
-    <row r="78">
+      <c r="I77" s="2" t="n"/>
+      <c r="J77" s="6" t="n"/>
+      <c r="K77" s="2" t="n"/>
+    </row>
+    <row r="78" ht="32" customHeight="1">
       <c r="A78" s="2" t="n"/>
       <c r="B78" s="3" t="n"/>
       <c r="C78" s="4" t="n"/>
@@ -1455,10 +1544,11 @@
       <c r="F78" s="2" t="n"/>
       <c r="G78" s="2" t="n"/>
       <c r="H78" s="5" t="n"/>
-      <c r="I78" s="6" t="n"/>
-      <c r="J78" s="7" t="n"/>
-    </row>
-    <row r="79">
+      <c r="I78" s="2" t="n"/>
+      <c r="J78" s="6" t="n"/>
+      <c r="K78" s="2" t="n"/>
+    </row>
+    <row r="79" ht="32" customHeight="1">
       <c r="A79" s="2" t="n"/>
       <c r="B79" s="3" t="n"/>
       <c r="C79" s="4" t="n"/>
@@ -1467,10 +1557,11 @@
       <c r="F79" s="2" t="n"/>
       <c r="G79" s="2" t="n"/>
       <c r="H79" s="5" t="n"/>
-      <c r="I79" s="6" t="n"/>
-      <c r="J79" s="7" t="n"/>
-    </row>
-    <row r="80">
+      <c r="I79" s="2" t="n"/>
+      <c r="J79" s="6" t="n"/>
+      <c r="K79" s="2" t="n"/>
+    </row>
+    <row r="80" ht="32" customHeight="1">
       <c r="A80" s="2" t="n"/>
       <c r="B80" s="3" t="n"/>
       <c r="C80" s="4" t="n"/>
@@ -1479,10 +1570,11 @@
       <c r="F80" s="2" t="n"/>
       <c r="G80" s="2" t="n"/>
       <c r="H80" s="5" t="n"/>
-      <c r="I80" s="6" t="n"/>
-      <c r="J80" s="7" t="n"/>
-    </row>
-    <row r="81">
+      <c r="I80" s="2" t="n"/>
+      <c r="J80" s="6" t="n"/>
+      <c r="K80" s="2" t="n"/>
+    </row>
+    <row r="81" ht="32" customHeight="1">
       <c r="A81" s="2" t="n"/>
       <c r="B81" s="3" t="n"/>
       <c r="C81" s="4" t="n"/>
@@ -1491,10 +1583,11 @@
       <c r="F81" s="2" t="n"/>
       <c r="G81" s="2" t="n"/>
       <c r="H81" s="5" t="n"/>
-      <c r="I81" s="6" t="n"/>
-      <c r="J81" s="7" t="n"/>
-    </row>
-    <row r="82">
+      <c r="I81" s="2" t="n"/>
+      <c r="J81" s="6" t="n"/>
+      <c r="K81" s="2" t="n"/>
+    </row>
+    <row r="82" ht="32" customHeight="1">
       <c r="A82" s="2" t="n"/>
       <c r="B82" s="3" t="n"/>
       <c r="C82" s="4" t="n"/>
@@ -1503,10 +1596,11 @@
       <c r="F82" s="2" t="n"/>
       <c r="G82" s="2" t="n"/>
       <c r="H82" s="5" t="n"/>
-      <c r="I82" s="6" t="n"/>
-      <c r="J82" s="7" t="n"/>
-    </row>
-    <row r="83">
+      <c r="I82" s="2" t="n"/>
+      <c r="J82" s="6" t="n"/>
+      <c r="K82" s="2" t="n"/>
+    </row>
+    <row r="83" ht="32" customHeight="1">
       <c r="A83" s="2" t="n"/>
       <c r="B83" s="3" t="n"/>
       <c r="C83" s="4" t="n"/>
@@ -1515,10 +1609,11 @@
       <c r="F83" s="2" t="n"/>
       <c r="G83" s="2" t="n"/>
       <c r="H83" s="5" t="n"/>
-      <c r="I83" s="6" t="n"/>
-      <c r="J83" s="7" t="n"/>
-    </row>
-    <row r="84">
+      <c r="I83" s="2" t="n"/>
+      <c r="J83" s="6" t="n"/>
+      <c r="K83" s="2" t="n"/>
+    </row>
+    <row r="84" ht="32" customHeight="1">
       <c r="A84" s="2" t="n"/>
       <c r="B84" s="3" t="n"/>
       <c r="C84" s="4" t="n"/>
@@ -1527,10 +1622,11 @@
       <c r="F84" s="2" t="n"/>
       <c r="G84" s="2" t="n"/>
       <c r="H84" s="5" t="n"/>
-      <c r="I84" s="6" t="n"/>
-      <c r="J84" s="7" t="n"/>
-    </row>
-    <row r="85">
+      <c r="I84" s="2" t="n"/>
+      <c r="J84" s="6" t="n"/>
+      <c r="K84" s="2" t="n"/>
+    </row>
+    <row r="85" ht="32" customHeight="1">
       <c r="A85" s="2" t="n"/>
       <c r="B85" s="3" t="n"/>
       <c r="C85" s="4" t="n"/>
@@ -1539,10 +1635,11 @@
       <c r="F85" s="2" t="n"/>
       <c r="G85" s="2" t="n"/>
       <c r="H85" s="5" t="n"/>
-      <c r="I85" s="6" t="n"/>
-      <c r="J85" s="7" t="n"/>
-    </row>
-    <row r="86">
+      <c r="I85" s="2" t="n"/>
+      <c r="J85" s="6" t="n"/>
+      <c r="K85" s="2" t="n"/>
+    </row>
+    <row r="86" ht="32" customHeight="1">
       <c r="A86" s="2" t="n"/>
       <c r="B86" s="3" t="n"/>
       <c r="C86" s="4" t="n"/>
@@ -1551,10 +1648,11 @@
       <c r="F86" s="2" t="n"/>
       <c r="G86" s="2" t="n"/>
       <c r="H86" s="5" t="n"/>
-      <c r="I86" s="6" t="n"/>
-      <c r="J86" s="7" t="n"/>
-    </row>
-    <row r="87">
+      <c r="I86" s="2" t="n"/>
+      <c r="J86" s="6" t="n"/>
+      <c r="K86" s="2" t="n"/>
+    </row>
+    <row r="87" ht="32" customHeight="1">
       <c r="A87" s="2" t="n"/>
       <c r="B87" s="3" t="n"/>
       <c r="C87" s="4" t="n"/>
@@ -1563,10 +1661,11 @@
       <c r="F87" s="2" t="n"/>
       <c r="G87" s="2" t="n"/>
       <c r="H87" s="5" t="n"/>
-      <c r="I87" s="6" t="n"/>
-      <c r="J87" s="7" t="n"/>
-    </row>
-    <row r="88">
+      <c r="I87" s="2" t="n"/>
+      <c r="J87" s="6" t="n"/>
+      <c r="K87" s="2" t="n"/>
+    </row>
+    <row r="88" ht="32" customHeight="1">
       <c r="A88" s="2" t="n"/>
       <c r="B88" s="3" t="n"/>
       <c r="C88" s="4" t="n"/>
@@ -1575,10 +1674,11 @@
       <c r="F88" s="2" t="n"/>
       <c r="G88" s="2" t="n"/>
       <c r="H88" s="5" t="n"/>
-      <c r="I88" s="6" t="n"/>
-      <c r="J88" s="7" t="n"/>
-    </row>
-    <row r="89">
+      <c r="I88" s="2" t="n"/>
+      <c r="J88" s="6" t="n"/>
+      <c r="K88" s="2" t="n"/>
+    </row>
+    <row r="89" ht="32" customHeight="1">
       <c r="A89" s="2" t="n"/>
       <c r="B89" s="3" t="n"/>
       <c r="C89" s="4" t="n"/>
@@ -1587,10 +1687,11 @@
       <c r="F89" s="2" t="n"/>
       <c r="G89" s="2" t="n"/>
       <c r="H89" s="5" t="n"/>
-      <c r="I89" s="6" t="n"/>
-      <c r="J89" s="7" t="n"/>
-    </row>
-    <row r="90">
+      <c r="I89" s="2" t="n"/>
+      <c r="J89" s="6" t="n"/>
+      <c r="K89" s="2" t="n"/>
+    </row>
+    <row r="90" ht="32" customHeight="1">
       <c r="A90" s="2" t="n"/>
       <c r="B90" s="3" t="n"/>
       <c r="C90" s="4" t="n"/>
@@ -1599,10 +1700,11 @@
       <c r="F90" s="2" t="n"/>
       <c r="G90" s="2" t="n"/>
       <c r="H90" s="5" t="n"/>
-      <c r="I90" s="6" t="n"/>
-      <c r="J90" s="7" t="n"/>
-    </row>
-    <row r="91">
+      <c r="I90" s="2" t="n"/>
+      <c r="J90" s="6" t="n"/>
+      <c r="K90" s="2" t="n"/>
+    </row>
+    <row r="91" ht="32" customHeight="1">
       <c r="A91" s="2" t="n"/>
       <c r="B91" s="3" t="n"/>
       <c r="C91" s="4" t="n"/>
@@ -1611,10 +1713,11 @@
       <c r="F91" s="2" t="n"/>
       <c r="G91" s="2" t="n"/>
       <c r="H91" s="5" t="n"/>
-      <c r="I91" s="6" t="n"/>
-      <c r="J91" s="7" t="n"/>
-    </row>
-    <row r="92">
+      <c r="I91" s="2" t="n"/>
+      <c r="J91" s="6" t="n"/>
+      <c r="K91" s="2" t="n"/>
+    </row>
+    <row r="92" ht="32" customHeight="1">
       <c r="A92" s="2" t="n"/>
       <c r="B92" s="3" t="n"/>
       <c r="C92" s="4" t="n"/>
@@ -1623,10 +1726,11 @@
       <c r="F92" s="2" t="n"/>
       <c r="G92" s="2" t="n"/>
       <c r="H92" s="5" t="n"/>
-      <c r="I92" s="6" t="n"/>
-      <c r="J92" s="7" t="n"/>
-    </row>
-    <row r="93">
+      <c r="I92" s="2" t="n"/>
+      <c r="J92" s="6" t="n"/>
+      <c r="K92" s="2" t="n"/>
+    </row>
+    <row r="93" ht="32" customHeight="1">
       <c r="A93" s="2" t="n"/>
       <c r="B93" s="3" t="n"/>
       <c r="C93" s="4" t="n"/>
@@ -1635,10 +1739,11 @@
       <c r="F93" s="2" t="n"/>
       <c r="G93" s="2" t="n"/>
       <c r="H93" s="5" t="n"/>
-      <c r="I93" s="6" t="n"/>
-      <c r="J93" s="7" t="n"/>
-    </row>
-    <row r="94">
+      <c r="I93" s="2" t="n"/>
+      <c r="J93" s="6" t="n"/>
+      <c r="K93" s="2" t="n"/>
+    </row>
+    <row r="94" ht="32" customHeight="1">
       <c r="A94" s="2" t="n"/>
       <c r="B94" s="3" t="n"/>
       <c r="C94" s="4" t="n"/>
@@ -1647,10 +1752,11 @@
       <c r="F94" s="2" t="n"/>
       <c r="G94" s="2" t="n"/>
       <c r="H94" s="5" t="n"/>
-      <c r="I94" s="6" t="n"/>
-      <c r="J94" s="7" t="n"/>
-    </row>
-    <row r="95">
+      <c r="I94" s="2" t="n"/>
+      <c r="J94" s="6" t="n"/>
+      <c r="K94" s="2" t="n"/>
+    </row>
+    <row r="95" ht="32" customHeight="1">
       <c r="A95" s="2" t="n"/>
       <c r="B95" s="3" t="n"/>
       <c r="C95" s="4" t="n"/>
@@ -1659,10 +1765,11 @@
       <c r="F95" s="2" t="n"/>
       <c r="G95" s="2" t="n"/>
       <c r="H95" s="5" t="n"/>
-      <c r="I95" s="6" t="n"/>
-      <c r="J95" s="7" t="n"/>
-    </row>
-    <row r="96">
+      <c r="I95" s="2" t="n"/>
+      <c r="J95" s="6" t="n"/>
+      <c r="K95" s="2" t="n"/>
+    </row>
+    <row r="96" ht="32" customHeight="1">
       <c r="A96" s="2" t="n"/>
       <c r="B96" s="3" t="n"/>
       <c r="C96" s="4" t="n"/>
@@ -1671,10 +1778,11 @@
       <c r="F96" s="2" t="n"/>
       <c r="G96" s="2" t="n"/>
       <c r="H96" s="5" t="n"/>
-      <c r="I96" s="6" t="n"/>
-      <c r="J96" s="7" t="n"/>
-    </row>
-    <row r="97">
+      <c r="I96" s="2" t="n"/>
+      <c r="J96" s="6" t="n"/>
+      <c r="K96" s="2" t="n"/>
+    </row>
+    <row r="97" ht="32" customHeight="1">
       <c r="A97" s="2" t="n"/>
       <c r="B97" s="3" t="n"/>
       <c r="C97" s="4" t="n"/>
@@ -1683,10 +1791,11 @@
       <c r="F97" s="2" t="n"/>
       <c r="G97" s="2" t="n"/>
       <c r="H97" s="5" t="n"/>
-      <c r="I97" s="6" t="n"/>
-      <c r="J97" s="7" t="n"/>
-    </row>
-    <row r="98">
+      <c r="I97" s="2" t="n"/>
+      <c r="J97" s="6" t="n"/>
+      <c r="K97" s="2" t="n"/>
+    </row>
+    <row r="98" ht="32" customHeight="1">
       <c r="A98" s="2" t="n"/>
       <c r="B98" s="3" t="n"/>
       <c r="C98" s="4" t="n"/>
@@ -1695,10 +1804,11 @@
       <c r="F98" s="2" t="n"/>
       <c r="G98" s="2" t="n"/>
       <c r="H98" s="5" t="n"/>
-      <c r="I98" s="6" t="n"/>
-      <c r="J98" s="7" t="n"/>
-    </row>
-    <row r="99">
+      <c r="I98" s="2" t="n"/>
+      <c r="J98" s="6" t="n"/>
+      <c r="K98" s="2" t="n"/>
+    </row>
+    <row r="99" ht="32" customHeight="1">
       <c r="A99" s="2" t="n"/>
       <c r="B99" s="3" t="n"/>
       <c r="C99" s="4" t="n"/>
@@ -1707,10 +1817,11 @@
       <c r="F99" s="2" t="n"/>
       <c r="G99" s="2" t="n"/>
       <c r="H99" s="5" t="n"/>
-      <c r="I99" s="6" t="n"/>
-      <c r="J99" s="7" t="n"/>
-    </row>
-    <row r="100">
+      <c r="I99" s="2" t="n"/>
+      <c r="J99" s="6" t="n"/>
+      <c r="K99" s="2" t="n"/>
+    </row>
+    <row r="100" ht="32" customHeight="1">
       <c r="A100" s="2" t="n"/>
       <c r="B100" s="3" t="n"/>
       <c r="C100" s="4" t="n"/>
@@ -1719,10 +1830,11 @@
       <c r="F100" s="2" t="n"/>
       <c r="G100" s="2" t="n"/>
       <c r="H100" s="5" t="n"/>
-      <c r="I100" s="6" t="n"/>
-      <c r="J100" s="7" t="n"/>
-    </row>
-    <row r="101">
+      <c r="I100" s="2" t="n"/>
+      <c r="J100" s="6" t="n"/>
+      <c r="K100" s="2" t="n"/>
+    </row>
+    <row r="101" ht="32" customHeight="1">
       <c r="A101" s="2" t="n"/>
       <c r="B101" s="3" t="n"/>
       <c r="C101" s="4" t="n"/>
@@ -1731,11 +1843,12 @@
       <c r="F101" s="2" t="n"/>
       <c r="G101" s="2" t="n"/>
       <c r="H101" s="5" t="n"/>
-      <c r="I101" s="6" t="n"/>
-      <c r="J101" s="7" t="n"/>
+      <c r="I101" s="2" t="n"/>
+      <c r="J101" s="6" t="n"/>
+      <c r="K101" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J101"/>
+  <autoFilter ref="A1:K101"/>
   <conditionalFormatting sqref="B2:I101">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>AND($A2&lt;&gt;"",B2="")</formula>

</xml_diff>

<commit_message>
Let availability rows auto-fit and widen column
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F2bKD8QwZtMnPmjESyq7MM
</commit_message>
<xml_diff>
--- a/DiscoverEU_KA155_Katilimci_Tablosu.xlsx
+++ b/DiscoverEU_KA155_Katilimci_Tablosu.xlsx
@@ -79,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -98,6 +98,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -486,7 +489,7 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="70" customWidth="1" min="10" max="10"/>
     <col width="30" customWidth="1" min="11" max="11"/>
     <col width="40" customWidth="1" min="12" max="12"/>
   </cols>
@@ -553,7 +556,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="32" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="n"/>
       <c r="B2" s="3" t="n"/>
       <c r="C2" s="4" t="n"/>
@@ -563,11 +566,11 @@
       <c r="G2" s="2" t="n"/>
       <c r="H2" s="2" t="n"/>
       <c r="I2" s="5" t="n"/>
-      <c r="J2" s="2" t="n"/>
+      <c r="J2" s="7" t="n"/>
       <c r="K2" s="6" t="n"/>
       <c r="L2" s="2" t="n"/>
     </row>
-    <row r="3" ht="32" customHeight="1">
+    <row r="3">
       <c r="A3" s="2" t="n"/>
       <c r="B3" s="3" t="n"/>
       <c r="C3" s="4" t="n"/>
@@ -577,11 +580,11 @@
       <c r="G3" s="2" t="n"/>
       <c r="H3" s="2" t="n"/>
       <c r="I3" s="5" t="n"/>
-      <c r="J3" s="2" t="n"/>
+      <c r="J3" s="7" t="n"/>
       <c r="K3" s="6" t="n"/>
       <c r="L3" s="2" t="n"/>
     </row>
-    <row r="4" ht="32" customHeight="1">
+    <row r="4">
       <c r="A4" s="2" t="n"/>
       <c r="B4" s="3" t="n"/>
       <c r="C4" s="4" t="n"/>
@@ -591,11 +594,11 @@
       <c r="G4" s="2" t="n"/>
       <c r="H4" s="2" t="n"/>
       <c r="I4" s="5" t="n"/>
-      <c r="J4" s="2" t="n"/>
+      <c r="J4" s="7" t="n"/>
       <c r="K4" s="6" t="n"/>
       <c r="L4" s="2" t="n"/>
     </row>
-    <row r="5" ht="32" customHeight="1">
+    <row r="5">
       <c r="A5" s="2" t="n"/>
       <c r="B5" s="3" t="n"/>
       <c r="C5" s="4" t="n"/>
@@ -605,11 +608,11 @@
       <c r="G5" s="2" t="n"/>
       <c r="H5" s="2" t="n"/>
       <c r="I5" s="5" t="n"/>
-      <c r="J5" s="2" t="n"/>
+      <c r="J5" s="7" t="n"/>
       <c r="K5" s="6" t="n"/>
       <c r="L5" s="2" t="n"/>
     </row>
-    <row r="6" ht="32" customHeight="1">
+    <row r="6">
       <c r="A6" s="2" t="n"/>
       <c r="B6" s="3" t="n"/>
       <c r="C6" s="4" t="n"/>
@@ -619,11 +622,11 @@
       <c r="G6" s="2" t="n"/>
       <c r="H6" s="2" t="n"/>
       <c r="I6" s="5" t="n"/>
-      <c r="J6" s="2" t="n"/>
+      <c r="J6" s="7" t="n"/>
       <c r="K6" s="6" t="n"/>
       <c r="L6" s="2" t="n"/>
     </row>
-    <row r="7" ht="32" customHeight="1">
+    <row r="7">
       <c r="A7" s="2" t="n"/>
       <c r="B7" s="3" t="n"/>
       <c r="C7" s="4" t="n"/>
@@ -633,11 +636,11 @@
       <c r="G7" s="2" t="n"/>
       <c r="H7" s="2" t="n"/>
       <c r="I7" s="5" t="n"/>
-      <c r="J7" s="2" t="n"/>
+      <c r="J7" s="7" t="n"/>
       <c r="K7" s="6" t="n"/>
       <c r="L7" s="2" t="n"/>
     </row>
-    <row r="8" ht="32" customHeight="1">
+    <row r="8">
       <c r="A8" s="2" t="n"/>
       <c r="B8" s="3" t="n"/>
       <c r="C8" s="4" t="n"/>
@@ -647,11 +650,11 @@
       <c r="G8" s="2" t="n"/>
       <c r="H8" s="2" t="n"/>
       <c r="I8" s="5" t="n"/>
-      <c r="J8" s="2" t="n"/>
+      <c r="J8" s="7" t="n"/>
       <c r="K8" s="6" t="n"/>
       <c r="L8" s="2" t="n"/>
     </row>
-    <row r="9" ht="32" customHeight="1">
+    <row r="9">
       <c r="A9" s="2" t="n"/>
       <c r="B9" s="3" t="n"/>
       <c r="C9" s="4" t="n"/>
@@ -661,11 +664,11 @@
       <c r="G9" s="2" t="n"/>
       <c r="H9" s="2" t="n"/>
       <c r="I9" s="5" t="n"/>
-      <c r="J9" s="2" t="n"/>
+      <c r="J9" s="7" t="n"/>
       <c r="K9" s="6" t="n"/>
       <c r="L9" s="2" t="n"/>
     </row>
-    <row r="10" ht="32" customHeight="1">
+    <row r="10">
       <c r="A10" s="2" t="n"/>
       <c r="B10" s="3" t="n"/>
       <c r="C10" s="4" t="n"/>
@@ -675,11 +678,11 @@
       <c r="G10" s="2" t="n"/>
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="5" t="n"/>
-      <c r="J10" s="2" t="n"/>
+      <c r="J10" s="7" t="n"/>
       <c r="K10" s="6" t="n"/>
       <c r="L10" s="2" t="n"/>
     </row>
-    <row r="11" ht="32" customHeight="1">
+    <row r="11">
       <c r="A11" s="2" t="n"/>
       <c r="B11" s="3" t="n"/>
       <c r="C11" s="4" t="n"/>
@@ -689,11 +692,11 @@
       <c r="G11" s="2" t="n"/>
       <c r="H11" s="2" t="n"/>
       <c r="I11" s="5" t="n"/>
-      <c r="J11" s="2" t="n"/>
+      <c r="J11" s="7" t="n"/>
       <c r="K11" s="6" t="n"/>
       <c r="L11" s="2" t="n"/>
     </row>
-    <row r="12" ht="32" customHeight="1">
+    <row r="12">
       <c r="A12" s="2" t="n"/>
       <c r="B12" s="3" t="n"/>
       <c r="C12" s="4" t="n"/>
@@ -703,11 +706,11 @@
       <c r="G12" s="2" t="n"/>
       <c r="H12" s="2" t="n"/>
       <c r="I12" s="5" t="n"/>
-      <c r="J12" s="2" t="n"/>
+      <c r="J12" s="7" t="n"/>
       <c r="K12" s="6" t="n"/>
       <c r="L12" s="2" t="n"/>
     </row>
-    <row r="13" ht="32" customHeight="1">
+    <row r="13">
       <c r="A13" s="2" t="n"/>
       <c r="B13" s="3" t="n"/>
       <c r="C13" s="4" t="n"/>
@@ -717,11 +720,11 @@
       <c r="G13" s="2" t="n"/>
       <c r="H13" s="2" t="n"/>
       <c r="I13" s="5" t="n"/>
-      <c r="J13" s="2" t="n"/>
+      <c r="J13" s="7" t="n"/>
       <c r="K13" s="6" t="n"/>
       <c r="L13" s="2" t="n"/>
     </row>
-    <row r="14" ht="32" customHeight="1">
+    <row r="14">
       <c r="A14" s="2" t="n"/>
       <c r="B14" s="3" t="n"/>
       <c r="C14" s="4" t="n"/>
@@ -731,11 +734,11 @@
       <c r="G14" s="2" t="n"/>
       <c r="H14" s="2" t="n"/>
       <c r="I14" s="5" t="n"/>
-      <c r="J14" s="2" t="n"/>
+      <c r="J14" s="7" t="n"/>
       <c r="K14" s="6" t="n"/>
       <c r="L14" s="2" t="n"/>
     </row>
-    <row r="15" ht="32" customHeight="1">
+    <row r="15">
       <c r="A15" s="2" t="n"/>
       <c r="B15" s="3" t="n"/>
       <c r="C15" s="4" t="n"/>
@@ -745,11 +748,11 @@
       <c r="G15" s="2" t="n"/>
       <c r="H15" s="2" t="n"/>
       <c r="I15" s="5" t="n"/>
-      <c r="J15" s="2" t="n"/>
+      <c r="J15" s="7" t="n"/>
       <c r="K15" s="6" t="n"/>
       <c r="L15" s="2" t="n"/>
     </row>
-    <row r="16" ht="32" customHeight="1">
+    <row r="16">
       <c r="A16" s="2" t="n"/>
       <c r="B16" s="3" t="n"/>
       <c r="C16" s="4" t="n"/>
@@ -759,11 +762,11 @@
       <c r="G16" s="2" t="n"/>
       <c r="H16" s="2" t="n"/>
       <c r="I16" s="5" t="n"/>
-      <c r="J16" s="2" t="n"/>
+      <c r="J16" s="7" t="n"/>
       <c r="K16" s="6" t="n"/>
       <c r="L16" s="2" t="n"/>
     </row>
-    <row r="17" ht="32" customHeight="1">
+    <row r="17">
       <c r="A17" s="2" t="n"/>
       <c r="B17" s="3" t="n"/>
       <c r="C17" s="4" t="n"/>
@@ -773,11 +776,11 @@
       <c r="G17" s="2" t="n"/>
       <c r="H17" s="2" t="n"/>
       <c r="I17" s="5" t="n"/>
-      <c r="J17" s="2" t="n"/>
+      <c r="J17" s="7" t="n"/>
       <c r="K17" s="6" t="n"/>
       <c r="L17" s="2" t="n"/>
     </row>
-    <row r="18" ht="32" customHeight="1">
+    <row r="18">
       <c r="A18" s="2" t="n"/>
       <c r="B18" s="3" t="n"/>
       <c r="C18" s="4" t="n"/>
@@ -787,11 +790,11 @@
       <c r="G18" s="2" t="n"/>
       <c r="H18" s="2" t="n"/>
       <c r="I18" s="5" t="n"/>
-      <c r="J18" s="2" t="n"/>
+      <c r="J18" s="7" t="n"/>
       <c r="K18" s="6" t="n"/>
       <c r="L18" s="2" t="n"/>
     </row>
-    <row r="19" ht="32" customHeight="1">
+    <row r="19">
       <c r="A19" s="2" t="n"/>
       <c r="B19" s="3" t="n"/>
       <c r="C19" s="4" t="n"/>
@@ -801,11 +804,11 @@
       <c r="G19" s="2" t="n"/>
       <c r="H19" s="2" t="n"/>
       <c r="I19" s="5" t="n"/>
-      <c r="J19" s="2" t="n"/>
+      <c r="J19" s="7" t="n"/>
       <c r="K19" s="6" t="n"/>
       <c r="L19" s="2" t="n"/>
     </row>
-    <row r="20" ht="32" customHeight="1">
+    <row r="20">
       <c r="A20" s="2" t="n"/>
       <c r="B20" s="3" t="n"/>
       <c r="C20" s="4" t="n"/>
@@ -815,11 +818,11 @@
       <c r="G20" s="2" t="n"/>
       <c r="H20" s="2" t="n"/>
       <c r="I20" s="5" t="n"/>
-      <c r="J20" s="2" t="n"/>
+      <c r="J20" s="7" t="n"/>
       <c r="K20" s="6" t="n"/>
       <c r="L20" s="2" t="n"/>
     </row>
-    <row r="21" ht="32" customHeight="1">
+    <row r="21">
       <c r="A21" s="2" t="n"/>
       <c r="B21" s="3" t="n"/>
       <c r="C21" s="4" t="n"/>
@@ -829,11 +832,11 @@
       <c r="G21" s="2" t="n"/>
       <c r="H21" s="2" t="n"/>
       <c r="I21" s="5" t="n"/>
-      <c r="J21" s="2" t="n"/>
+      <c r="J21" s="7" t="n"/>
       <c r="K21" s="6" t="n"/>
       <c r="L21" s="2" t="n"/>
     </row>
-    <row r="22" ht="32" customHeight="1">
+    <row r="22">
       <c r="A22" s="2" t="n"/>
       <c r="B22" s="3" t="n"/>
       <c r="C22" s="4" t="n"/>
@@ -843,11 +846,11 @@
       <c r="G22" s="2" t="n"/>
       <c r="H22" s="2" t="n"/>
       <c r="I22" s="5" t="n"/>
-      <c r="J22" s="2" t="n"/>
+      <c r="J22" s="7" t="n"/>
       <c r="K22" s="6" t="n"/>
       <c r="L22" s="2" t="n"/>
     </row>
-    <row r="23" ht="32" customHeight="1">
+    <row r="23">
       <c r="A23" s="2" t="n"/>
       <c r="B23" s="3" t="n"/>
       <c r="C23" s="4" t="n"/>
@@ -857,11 +860,11 @@
       <c r="G23" s="2" t="n"/>
       <c r="H23" s="2" t="n"/>
       <c r="I23" s="5" t="n"/>
-      <c r="J23" s="2" t="n"/>
+      <c r="J23" s="7" t="n"/>
       <c r="K23" s="6" t="n"/>
       <c r="L23" s="2" t="n"/>
     </row>
-    <row r="24" ht="32" customHeight="1">
+    <row r="24">
       <c r="A24" s="2" t="n"/>
       <c r="B24" s="3" t="n"/>
       <c r="C24" s="4" t="n"/>
@@ -871,11 +874,11 @@
       <c r="G24" s="2" t="n"/>
       <c r="H24" s="2" t="n"/>
       <c r="I24" s="5" t="n"/>
-      <c r="J24" s="2" t="n"/>
+      <c r="J24" s="7" t="n"/>
       <c r="K24" s="6" t="n"/>
       <c r="L24" s="2" t="n"/>
     </row>
-    <row r="25" ht="32" customHeight="1">
+    <row r="25">
       <c r="A25" s="2" t="n"/>
       <c r="B25" s="3" t="n"/>
       <c r="C25" s="4" t="n"/>
@@ -885,11 +888,11 @@
       <c r="G25" s="2" t="n"/>
       <c r="H25" s="2" t="n"/>
       <c r="I25" s="5" t="n"/>
-      <c r="J25" s="2" t="n"/>
+      <c r="J25" s="7" t="n"/>
       <c r="K25" s="6" t="n"/>
       <c r="L25" s="2" t="n"/>
     </row>
-    <row r="26" ht="32" customHeight="1">
+    <row r="26">
       <c r="A26" s="2" t="n"/>
       <c r="B26" s="3" t="n"/>
       <c r="C26" s="4" t="n"/>
@@ -899,11 +902,11 @@
       <c r="G26" s="2" t="n"/>
       <c r="H26" s="2" t="n"/>
       <c r="I26" s="5" t="n"/>
-      <c r="J26" s="2" t="n"/>
+      <c r="J26" s="7" t="n"/>
       <c r="K26" s="6" t="n"/>
       <c r="L26" s="2" t="n"/>
     </row>
-    <row r="27" ht="32" customHeight="1">
+    <row r="27">
       <c r="A27" s="2" t="n"/>
       <c r="B27" s="3" t="n"/>
       <c r="C27" s="4" t="n"/>
@@ -913,11 +916,11 @@
       <c r="G27" s="2" t="n"/>
       <c r="H27" s="2" t="n"/>
       <c r="I27" s="5" t="n"/>
-      <c r="J27" s="2" t="n"/>
+      <c r="J27" s="7" t="n"/>
       <c r="K27" s="6" t="n"/>
       <c r="L27" s="2" t="n"/>
     </row>
-    <row r="28" ht="32" customHeight="1">
+    <row r="28">
       <c r="A28" s="2" t="n"/>
       <c r="B28" s="3" t="n"/>
       <c r="C28" s="4" t="n"/>
@@ -927,11 +930,11 @@
       <c r="G28" s="2" t="n"/>
       <c r="H28" s="2" t="n"/>
       <c r="I28" s="5" t="n"/>
-      <c r="J28" s="2" t="n"/>
+      <c r="J28" s="7" t="n"/>
       <c r="K28" s="6" t="n"/>
       <c r="L28" s="2" t="n"/>
     </row>
-    <row r="29" ht="32" customHeight="1">
+    <row r="29">
       <c r="A29" s="2" t="n"/>
       <c r="B29" s="3" t="n"/>
       <c r="C29" s="4" t="n"/>
@@ -941,11 +944,11 @@
       <c r="G29" s="2" t="n"/>
       <c r="H29" s="2" t="n"/>
       <c r="I29" s="5" t="n"/>
-      <c r="J29" s="2" t="n"/>
+      <c r="J29" s="7" t="n"/>
       <c r="K29" s="6" t="n"/>
       <c r="L29" s="2" t="n"/>
     </row>
-    <row r="30" ht="32" customHeight="1">
+    <row r="30">
       <c r="A30" s="2" t="n"/>
       <c r="B30" s="3" t="n"/>
       <c r="C30" s="4" t="n"/>
@@ -955,11 +958,11 @@
       <c r="G30" s="2" t="n"/>
       <c r="H30" s="2" t="n"/>
       <c r="I30" s="5" t="n"/>
-      <c r="J30" s="2" t="n"/>
+      <c r="J30" s="7" t="n"/>
       <c r="K30" s="6" t="n"/>
       <c r="L30" s="2" t="n"/>
     </row>
-    <row r="31" ht="32" customHeight="1">
+    <row r="31">
       <c r="A31" s="2" t="n"/>
       <c r="B31" s="3" t="n"/>
       <c r="C31" s="4" t="n"/>
@@ -969,11 +972,11 @@
       <c r="G31" s="2" t="n"/>
       <c r="H31" s="2" t="n"/>
       <c r="I31" s="5" t="n"/>
-      <c r="J31" s="2" t="n"/>
+      <c r="J31" s="7" t="n"/>
       <c r="K31" s="6" t="n"/>
       <c r="L31" s="2" t="n"/>
     </row>
-    <row r="32" ht="32" customHeight="1">
+    <row r="32">
       <c r="A32" s="2" t="n"/>
       <c r="B32" s="3" t="n"/>
       <c r="C32" s="4" t="n"/>
@@ -983,11 +986,11 @@
       <c r="G32" s="2" t="n"/>
       <c r="H32" s="2" t="n"/>
       <c r="I32" s="5" t="n"/>
-      <c r="J32" s="2" t="n"/>
+      <c r="J32" s="7" t="n"/>
       <c r="K32" s="6" t="n"/>
       <c r="L32" s="2" t="n"/>
     </row>
-    <row r="33" ht="32" customHeight="1">
+    <row r="33">
       <c r="A33" s="2" t="n"/>
       <c r="B33" s="3" t="n"/>
       <c r="C33" s="4" t="n"/>
@@ -997,11 +1000,11 @@
       <c r="G33" s="2" t="n"/>
       <c r="H33" s="2" t="n"/>
       <c r="I33" s="5" t="n"/>
-      <c r="J33" s="2" t="n"/>
+      <c r="J33" s="7" t="n"/>
       <c r="K33" s="6" t="n"/>
       <c r="L33" s="2" t="n"/>
     </row>
-    <row r="34" ht="32" customHeight="1">
+    <row r="34">
       <c r="A34" s="2" t="n"/>
       <c r="B34" s="3" t="n"/>
       <c r="C34" s="4" t="n"/>
@@ -1011,11 +1014,11 @@
       <c r="G34" s="2" t="n"/>
       <c r="H34" s="2" t="n"/>
       <c r="I34" s="5" t="n"/>
-      <c r="J34" s="2" t="n"/>
+      <c r="J34" s="7" t="n"/>
       <c r="K34" s="6" t="n"/>
       <c r="L34" s="2" t="n"/>
     </row>
-    <row r="35" ht="32" customHeight="1">
+    <row r="35">
       <c r="A35" s="2" t="n"/>
       <c r="B35" s="3" t="n"/>
       <c r="C35" s="4" t="n"/>
@@ -1025,11 +1028,11 @@
       <c r="G35" s="2" t="n"/>
       <c r="H35" s="2" t="n"/>
       <c r="I35" s="5" t="n"/>
-      <c r="J35" s="2" t="n"/>
+      <c r="J35" s="7" t="n"/>
       <c r="K35" s="6" t="n"/>
       <c r="L35" s="2" t="n"/>
     </row>
-    <row r="36" ht="32" customHeight="1">
+    <row r="36">
       <c r="A36" s="2" t="n"/>
       <c r="B36" s="3" t="n"/>
       <c r="C36" s="4" t="n"/>
@@ -1039,11 +1042,11 @@
       <c r="G36" s="2" t="n"/>
       <c r="H36" s="2" t="n"/>
       <c r="I36" s="5" t="n"/>
-      <c r="J36" s="2" t="n"/>
+      <c r="J36" s="7" t="n"/>
       <c r="K36" s="6" t="n"/>
       <c r="L36" s="2" t="n"/>
     </row>
-    <row r="37" ht="32" customHeight="1">
+    <row r="37">
       <c r="A37" s="2" t="n"/>
       <c r="B37" s="3" t="n"/>
       <c r="C37" s="4" t="n"/>
@@ -1053,11 +1056,11 @@
       <c r="G37" s="2" t="n"/>
       <c r="H37" s="2" t="n"/>
       <c r="I37" s="5" t="n"/>
-      <c r="J37" s="2" t="n"/>
+      <c r="J37" s="7" t="n"/>
       <c r="K37" s="6" t="n"/>
       <c r="L37" s="2" t="n"/>
     </row>
-    <row r="38" ht="32" customHeight="1">
+    <row r="38">
       <c r="A38" s="2" t="n"/>
       <c r="B38" s="3" t="n"/>
       <c r="C38" s="4" t="n"/>
@@ -1067,11 +1070,11 @@
       <c r="G38" s="2" t="n"/>
       <c r="H38" s="2" t="n"/>
       <c r="I38" s="5" t="n"/>
-      <c r="J38" s="2" t="n"/>
+      <c r="J38" s="7" t="n"/>
       <c r="K38" s="6" t="n"/>
       <c r="L38" s="2" t="n"/>
     </row>
-    <row r="39" ht="32" customHeight="1">
+    <row r="39">
       <c r="A39" s="2" t="n"/>
       <c r="B39" s="3" t="n"/>
       <c r="C39" s="4" t="n"/>
@@ -1081,11 +1084,11 @@
       <c r="G39" s="2" t="n"/>
       <c r="H39" s="2" t="n"/>
       <c r="I39" s="5" t="n"/>
-      <c r="J39" s="2" t="n"/>
+      <c r="J39" s="7" t="n"/>
       <c r="K39" s="6" t="n"/>
       <c r="L39" s="2" t="n"/>
     </row>
-    <row r="40" ht="32" customHeight="1">
+    <row r="40">
       <c r="A40" s="2" t="n"/>
       <c r="B40" s="3" t="n"/>
       <c r="C40" s="4" t="n"/>
@@ -1095,11 +1098,11 @@
       <c r="G40" s="2" t="n"/>
       <c r="H40" s="2" t="n"/>
       <c r="I40" s="5" t="n"/>
-      <c r="J40" s="2" t="n"/>
+      <c r="J40" s="7" t="n"/>
       <c r="K40" s="6" t="n"/>
       <c r="L40" s="2" t="n"/>
     </row>
-    <row r="41" ht="32" customHeight="1">
+    <row r="41">
       <c r="A41" s="2" t="n"/>
       <c r="B41" s="3" t="n"/>
       <c r="C41" s="4" t="n"/>
@@ -1109,11 +1112,11 @@
       <c r="G41" s="2" t="n"/>
       <c r="H41" s="2" t="n"/>
       <c r="I41" s="5" t="n"/>
-      <c r="J41" s="2" t="n"/>
+      <c r="J41" s="7" t="n"/>
       <c r="K41" s="6" t="n"/>
       <c r="L41" s="2" t="n"/>
     </row>
-    <row r="42" ht="32" customHeight="1">
+    <row r="42">
       <c r="A42" s="2" t="n"/>
       <c r="B42" s="3" t="n"/>
       <c r="C42" s="4" t="n"/>
@@ -1123,11 +1126,11 @@
       <c r="G42" s="2" t="n"/>
       <c r="H42" s="2" t="n"/>
       <c r="I42" s="5" t="n"/>
-      <c r="J42" s="2" t="n"/>
+      <c r="J42" s="7" t="n"/>
       <c r="K42" s="6" t="n"/>
       <c r="L42" s="2" t="n"/>
     </row>
-    <row r="43" ht="32" customHeight="1">
+    <row r="43">
       <c r="A43" s="2" t="n"/>
       <c r="B43" s="3" t="n"/>
       <c r="C43" s="4" t="n"/>
@@ -1137,11 +1140,11 @@
       <c r="G43" s="2" t="n"/>
       <c r="H43" s="2" t="n"/>
       <c r="I43" s="5" t="n"/>
-      <c r="J43" s="2" t="n"/>
+      <c r="J43" s="7" t="n"/>
       <c r="K43" s="6" t="n"/>
       <c r="L43" s="2" t="n"/>
     </row>
-    <row r="44" ht="32" customHeight="1">
+    <row r="44">
       <c r="A44" s="2" t="n"/>
       <c r="B44" s="3" t="n"/>
       <c r="C44" s="4" t="n"/>
@@ -1151,11 +1154,11 @@
       <c r="G44" s="2" t="n"/>
       <c r="H44" s="2" t="n"/>
       <c r="I44" s="5" t="n"/>
-      <c r="J44" s="2" t="n"/>
+      <c r="J44" s="7" t="n"/>
       <c r="K44" s="6" t="n"/>
       <c r="L44" s="2" t="n"/>
     </row>
-    <row r="45" ht="32" customHeight="1">
+    <row r="45">
       <c r="A45" s="2" t="n"/>
       <c r="B45" s="3" t="n"/>
       <c r="C45" s="4" t="n"/>
@@ -1165,11 +1168,11 @@
       <c r="G45" s="2" t="n"/>
       <c r="H45" s="2" t="n"/>
       <c r="I45" s="5" t="n"/>
-      <c r="J45" s="2" t="n"/>
+      <c r="J45" s="7" t="n"/>
       <c r="K45" s="6" t="n"/>
       <c r="L45" s="2" t="n"/>
     </row>
-    <row r="46" ht="32" customHeight="1">
+    <row r="46">
       <c r="A46" s="2" t="n"/>
       <c r="B46" s="3" t="n"/>
       <c r="C46" s="4" t="n"/>
@@ -1179,11 +1182,11 @@
       <c r="G46" s="2" t="n"/>
       <c r="H46" s="2" t="n"/>
       <c r="I46" s="5" t="n"/>
-      <c r="J46" s="2" t="n"/>
+      <c r="J46" s="7" t="n"/>
       <c r="K46" s="6" t="n"/>
       <c r="L46" s="2" t="n"/>
     </row>
-    <row r="47" ht="32" customHeight="1">
+    <row r="47">
       <c r="A47" s="2" t="n"/>
       <c r="B47" s="3" t="n"/>
       <c r="C47" s="4" t="n"/>
@@ -1193,11 +1196,11 @@
       <c r="G47" s="2" t="n"/>
       <c r="H47" s="2" t="n"/>
       <c r="I47" s="5" t="n"/>
-      <c r="J47" s="2" t="n"/>
+      <c r="J47" s="7" t="n"/>
       <c r="K47" s="6" t="n"/>
       <c r="L47" s="2" t="n"/>
     </row>
-    <row r="48" ht="32" customHeight="1">
+    <row r="48">
       <c r="A48" s="2" t="n"/>
       <c r="B48" s="3" t="n"/>
       <c r="C48" s="4" t="n"/>
@@ -1207,11 +1210,11 @@
       <c r="G48" s="2" t="n"/>
       <c r="H48" s="2" t="n"/>
       <c r="I48" s="5" t="n"/>
-      <c r="J48" s="2" t="n"/>
+      <c r="J48" s="7" t="n"/>
       <c r="K48" s="6" t="n"/>
       <c r="L48" s="2" t="n"/>
     </row>
-    <row r="49" ht="32" customHeight="1">
+    <row r="49">
       <c r="A49" s="2" t="n"/>
       <c r="B49" s="3" t="n"/>
       <c r="C49" s="4" t="n"/>
@@ -1221,11 +1224,11 @@
       <c r="G49" s="2" t="n"/>
       <c r="H49" s="2" t="n"/>
       <c r="I49" s="5" t="n"/>
-      <c r="J49" s="2" t="n"/>
+      <c r="J49" s="7" t="n"/>
       <c r="K49" s="6" t="n"/>
       <c r="L49" s="2" t="n"/>
     </row>
-    <row r="50" ht="32" customHeight="1">
+    <row r="50">
       <c r="A50" s="2" t="n"/>
       <c r="B50" s="3" t="n"/>
       <c r="C50" s="4" t="n"/>
@@ -1235,11 +1238,11 @@
       <c r="G50" s="2" t="n"/>
       <c r="H50" s="2" t="n"/>
       <c r="I50" s="5" t="n"/>
-      <c r="J50" s="2" t="n"/>
+      <c r="J50" s="7" t="n"/>
       <c r="K50" s="6" t="n"/>
       <c r="L50" s="2" t="n"/>
     </row>
-    <row r="51" ht="32" customHeight="1">
+    <row r="51">
       <c r="A51" s="2" t="n"/>
       <c r="B51" s="3" t="n"/>
       <c r="C51" s="4" t="n"/>
@@ -1249,11 +1252,11 @@
       <c r="G51" s="2" t="n"/>
       <c r="H51" s="2" t="n"/>
       <c r="I51" s="5" t="n"/>
-      <c r="J51" s="2" t="n"/>
+      <c r="J51" s="7" t="n"/>
       <c r="K51" s="6" t="n"/>
       <c r="L51" s="2" t="n"/>
     </row>
-    <row r="52" ht="32" customHeight="1">
+    <row r="52">
       <c r="A52" s="2" t="n"/>
       <c r="B52" s="3" t="n"/>
       <c r="C52" s="4" t="n"/>
@@ -1263,11 +1266,11 @@
       <c r="G52" s="2" t="n"/>
       <c r="H52" s="2" t="n"/>
       <c r="I52" s="5" t="n"/>
-      <c r="J52" s="2" t="n"/>
+      <c r="J52" s="7" t="n"/>
       <c r="K52" s="6" t="n"/>
       <c r="L52" s="2" t="n"/>
     </row>
-    <row r="53" ht="32" customHeight="1">
+    <row r="53">
       <c r="A53" s="2" t="n"/>
       <c r="B53" s="3" t="n"/>
       <c r="C53" s="4" t="n"/>
@@ -1277,11 +1280,11 @@
       <c r="G53" s="2" t="n"/>
       <c r="H53" s="2" t="n"/>
       <c r="I53" s="5" t="n"/>
-      <c r="J53" s="2" t="n"/>
+      <c r="J53" s="7" t="n"/>
       <c r="K53" s="6" t="n"/>
       <c r="L53" s="2" t="n"/>
     </row>
-    <row r="54" ht="32" customHeight="1">
+    <row r="54">
       <c r="A54" s="2" t="n"/>
       <c r="B54" s="3" t="n"/>
       <c r="C54" s="4" t="n"/>
@@ -1291,11 +1294,11 @@
       <c r="G54" s="2" t="n"/>
       <c r="H54" s="2" t="n"/>
       <c r="I54" s="5" t="n"/>
-      <c r="J54" s="2" t="n"/>
+      <c r="J54" s="7" t="n"/>
       <c r="K54" s="6" t="n"/>
       <c r="L54" s="2" t="n"/>
     </row>
-    <row r="55" ht="32" customHeight="1">
+    <row r="55">
       <c r="A55" s="2" t="n"/>
       <c r="B55" s="3" t="n"/>
       <c r="C55" s="4" t="n"/>
@@ -1305,11 +1308,11 @@
       <c r="G55" s="2" t="n"/>
       <c r="H55" s="2" t="n"/>
       <c r="I55" s="5" t="n"/>
-      <c r="J55" s="2" t="n"/>
+      <c r="J55" s="7" t="n"/>
       <c r="K55" s="6" t="n"/>
       <c r="L55" s="2" t="n"/>
     </row>
-    <row r="56" ht="32" customHeight="1">
+    <row r="56">
       <c r="A56" s="2" t="n"/>
       <c r="B56" s="3" t="n"/>
       <c r="C56" s="4" t="n"/>
@@ -1319,11 +1322,11 @@
       <c r="G56" s="2" t="n"/>
       <c r="H56" s="2" t="n"/>
       <c r="I56" s="5" t="n"/>
-      <c r="J56" s="2" t="n"/>
+      <c r="J56" s="7" t="n"/>
       <c r="K56" s="6" t="n"/>
       <c r="L56" s="2" t="n"/>
     </row>
-    <row r="57" ht="32" customHeight="1">
+    <row r="57">
       <c r="A57" s="2" t="n"/>
       <c r="B57" s="3" t="n"/>
       <c r="C57" s="4" t="n"/>
@@ -1333,11 +1336,11 @@
       <c r="G57" s="2" t="n"/>
       <c r="H57" s="2" t="n"/>
       <c r="I57" s="5" t="n"/>
-      <c r="J57" s="2" t="n"/>
+      <c r="J57" s="7" t="n"/>
       <c r="K57" s="6" t="n"/>
       <c r="L57" s="2" t="n"/>
     </row>
-    <row r="58" ht="32" customHeight="1">
+    <row r="58">
       <c r="A58" s="2" t="n"/>
       <c r="B58" s="3" t="n"/>
       <c r="C58" s="4" t="n"/>
@@ -1347,11 +1350,11 @@
       <c r="G58" s="2" t="n"/>
       <c r="H58" s="2" t="n"/>
       <c r="I58" s="5" t="n"/>
-      <c r="J58" s="2" t="n"/>
+      <c r="J58" s="7" t="n"/>
       <c r="K58" s="6" t="n"/>
       <c r="L58" s="2" t="n"/>
     </row>
-    <row r="59" ht="32" customHeight="1">
+    <row r="59">
       <c r="A59" s="2" t="n"/>
       <c r="B59" s="3" t="n"/>
       <c r="C59" s="4" t="n"/>
@@ -1361,11 +1364,11 @@
       <c r="G59" s="2" t="n"/>
       <c r="H59" s="2" t="n"/>
       <c r="I59" s="5" t="n"/>
-      <c r="J59" s="2" t="n"/>
+      <c r="J59" s="7" t="n"/>
       <c r="K59" s="6" t="n"/>
       <c r="L59" s="2" t="n"/>
     </row>
-    <row r="60" ht="32" customHeight="1">
+    <row r="60">
       <c r="A60" s="2" t="n"/>
       <c r="B60" s="3" t="n"/>
       <c r="C60" s="4" t="n"/>
@@ -1375,11 +1378,11 @@
       <c r="G60" s="2" t="n"/>
       <c r="H60" s="2" t="n"/>
       <c r="I60" s="5" t="n"/>
-      <c r="J60" s="2" t="n"/>
+      <c r="J60" s="7" t="n"/>
       <c r="K60" s="6" t="n"/>
       <c r="L60" s="2" t="n"/>
     </row>
-    <row r="61" ht="32" customHeight="1">
+    <row r="61">
       <c r="A61" s="2" t="n"/>
       <c r="B61" s="3" t="n"/>
       <c r="C61" s="4" t="n"/>
@@ -1389,11 +1392,11 @@
       <c r="G61" s="2" t="n"/>
       <c r="H61" s="2" t="n"/>
       <c r="I61" s="5" t="n"/>
-      <c r="J61" s="2" t="n"/>
+      <c r="J61" s="7" t="n"/>
       <c r="K61" s="6" t="n"/>
       <c r="L61" s="2" t="n"/>
     </row>
-    <row r="62" ht="32" customHeight="1">
+    <row r="62">
       <c r="A62" s="2" t="n"/>
       <c r="B62" s="3" t="n"/>
       <c r="C62" s="4" t="n"/>
@@ -1403,11 +1406,11 @@
       <c r="G62" s="2" t="n"/>
       <c r="H62" s="2" t="n"/>
       <c r="I62" s="5" t="n"/>
-      <c r="J62" s="2" t="n"/>
+      <c r="J62" s="7" t="n"/>
       <c r="K62" s="6" t="n"/>
       <c r="L62" s="2" t="n"/>
     </row>
-    <row r="63" ht="32" customHeight="1">
+    <row r="63">
       <c r="A63" s="2" t="n"/>
       <c r="B63" s="3" t="n"/>
       <c r="C63" s="4" t="n"/>
@@ -1417,11 +1420,11 @@
       <c r="G63" s="2" t="n"/>
       <c r="H63" s="2" t="n"/>
       <c r="I63" s="5" t="n"/>
-      <c r="J63" s="2" t="n"/>
+      <c r="J63" s="7" t="n"/>
       <c r="K63" s="6" t="n"/>
       <c r="L63" s="2" t="n"/>
     </row>
-    <row r="64" ht="32" customHeight="1">
+    <row r="64">
       <c r="A64" s="2" t="n"/>
       <c r="B64" s="3" t="n"/>
       <c r="C64" s="4" t="n"/>
@@ -1431,11 +1434,11 @@
       <c r="G64" s="2" t="n"/>
       <c r="H64" s="2" t="n"/>
       <c r="I64" s="5" t="n"/>
-      <c r="J64" s="2" t="n"/>
+      <c r="J64" s="7" t="n"/>
       <c r="K64" s="6" t="n"/>
       <c r="L64" s="2" t="n"/>
     </row>
-    <row r="65" ht="32" customHeight="1">
+    <row r="65">
       <c r="A65" s="2" t="n"/>
       <c r="B65" s="3" t="n"/>
       <c r="C65" s="4" t="n"/>
@@ -1445,11 +1448,11 @@
       <c r="G65" s="2" t="n"/>
       <c r="H65" s="2" t="n"/>
       <c r="I65" s="5" t="n"/>
-      <c r="J65" s="2" t="n"/>
+      <c r="J65" s="7" t="n"/>
       <c r="K65" s="6" t="n"/>
       <c r="L65" s="2" t="n"/>
     </row>
-    <row r="66" ht="32" customHeight="1">
+    <row r="66">
       <c r="A66" s="2" t="n"/>
       <c r="B66" s="3" t="n"/>
       <c r="C66" s="4" t="n"/>
@@ -1459,11 +1462,11 @@
       <c r="G66" s="2" t="n"/>
       <c r="H66" s="2" t="n"/>
       <c r="I66" s="5" t="n"/>
-      <c r="J66" s="2" t="n"/>
+      <c r="J66" s="7" t="n"/>
       <c r="K66" s="6" t="n"/>
       <c r="L66" s="2" t="n"/>
     </row>
-    <row r="67" ht="32" customHeight="1">
+    <row r="67">
       <c r="A67" s="2" t="n"/>
       <c r="B67" s="3" t="n"/>
       <c r="C67" s="4" t="n"/>
@@ -1473,11 +1476,11 @@
       <c r="G67" s="2" t="n"/>
       <c r="H67" s="2" t="n"/>
       <c r="I67" s="5" t="n"/>
-      <c r="J67" s="2" t="n"/>
+      <c r="J67" s="7" t="n"/>
       <c r="K67" s="6" t="n"/>
       <c r="L67" s="2" t="n"/>
     </row>
-    <row r="68" ht="32" customHeight="1">
+    <row r="68">
       <c r="A68" s="2" t="n"/>
       <c r="B68" s="3" t="n"/>
       <c r="C68" s="4" t="n"/>
@@ -1487,11 +1490,11 @@
       <c r="G68" s="2" t="n"/>
       <c r="H68" s="2" t="n"/>
       <c r="I68" s="5" t="n"/>
-      <c r="J68" s="2" t="n"/>
+      <c r="J68" s="7" t="n"/>
       <c r="K68" s="6" t="n"/>
       <c r="L68" s="2" t="n"/>
     </row>
-    <row r="69" ht="32" customHeight="1">
+    <row r="69">
       <c r="A69" s="2" t="n"/>
       <c r="B69" s="3" t="n"/>
       <c r="C69" s="4" t="n"/>
@@ -1501,11 +1504,11 @@
       <c r="G69" s="2" t="n"/>
       <c r="H69" s="2" t="n"/>
       <c r="I69" s="5" t="n"/>
-      <c r="J69" s="2" t="n"/>
+      <c r="J69" s="7" t="n"/>
       <c r="K69" s="6" t="n"/>
       <c r="L69" s="2" t="n"/>
     </row>
-    <row r="70" ht="32" customHeight="1">
+    <row r="70">
       <c r="A70" s="2" t="n"/>
       <c r="B70" s="3" t="n"/>
       <c r="C70" s="4" t="n"/>
@@ -1515,11 +1518,11 @@
       <c r="G70" s="2" t="n"/>
       <c r="H70" s="2" t="n"/>
       <c r="I70" s="5" t="n"/>
-      <c r="J70" s="2" t="n"/>
+      <c r="J70" s="7" t="n"/>
       <c r="K70" s="6" t="n"/>
       <c r="L70" s="2" t="n"/>
     </row>
-    <row r="71" ht="32" customHeight="1">
+    <row r="71">
       <c r="A71" s="2" t="n"/>
       <c r="B71" s="3" t="n"/>
       <c r="C71" s="4" t="n"/>
@@ -1529,11 +1532,11 @@
       <c r="G71" s="2" t="n"/>
       <c r="H71" s="2" t="n"/>
       <c r="I71" s="5" t="n"/>
-      <c r="J71" s="2" t="n"/>
+      <c r="J71" s="7" t="n"/>
       <c r="K71" s="6" t="n"/>
       <c r="L71" s="2" t="n"/>
     </row>
-    <row r="72" ht="32" customHeight="1">
+    <row r="72">
       <c r="A72" s="2" t="n"/>
       <c r="B72" s="3" t="n"/>
       <c r="C72" s="4" t="n"/>
@@ -1543,11 +1546,11 @@
       <c r="G72" s="2" t="n"/>
       <c r="H72" s="2" t="n"/>
       <c r="I72" s="5" t="n"/>
-      <c r="J72" s="2" t="n"/>
+      <c r="J72" s="7" t="n"/>
       <c r="K72" s="6" t="n"/>
       <c r="L72" s="2" t="n"/>
     </row>
-    <row r="73" ht="32" customHeight="1">
+    <row r="73">
       <c r="A73" s="2" t="n"/>
       <c r="B73" s="3" t="n"/>
       <c r="C73" s="4" t="n"/>
@@ -1557,11 +1560,11 @@
       <c r="G73" s="2" t="n"/>
       <c r="H73" s="2" t="n"/>
       <c r="I73" s="5" t="n"/>
-      <c r="J73" s="2" t="n"/>
+      <c r="J73" s="7" t="n"/>
       <c r="K73" s="6" t="n"/>
       <c r="L73" s="2" t="n"/>
     </row>
-    <row r="74" ht="32" customHeight="1">
+    <row r="74">
       <c r="A74" s="2" t="n"/>
       <c r="B74" s="3" t="n"/>
       <c r="C74" s="4" t="n"/>
@@ -1571,11 +1574,11 @@
       <c r="G74" s="2" t="n"/>
       <c r="H74" s="2" t="n"/>
       <c r="I74" s="5" t="n"/>
-      <c r="J74" s="2" t="n"/>
+      <c r="J74" s="7" t="n"/>
       <c r="K74" s="6" t="n"/>
       <c r="L74" s="2" t="n"/>
     </row>
-    <row r="75" ht="32" customHeight="1">
+    <row r="75">
       <c r="A75" s="2" t="n"/>
       <c r="B75" s="3" t="n"/>
       <c r="C75" s="4" t="n"/>
@@ -1585,11 +1588,11 @@
       <c r="G75" s="2" t="n"/>
       <c r="H75" s="2" t="n"/>
       <c r="I75" s="5" t="n"/>
-      <c r="J75" s="2" t="n"/>
+      <c r="J75" s="7" t="n"/>
       <c r="K75" s="6" t="n"/>
       <c r="L75" s="2" t="n"/>
     </row>
-    <row r="76" ht="32" customHeight="1">
+    <row r="76">
       <c r="A76" s="2" t="n"/>
       <c r="B76" s="3" t="n"/>
       <c r="C76" s="4" t="n"/>
@@ -1599,11 +1602,11 @@
       <c r="G76" s="2" t="n"/>
       <c r="H76" s="2" t="n"/>
       <c r="I76" s="5" t="n"/>
-      <c r="J76" s="2" t="n"/>
+      <c r="J76" s="7" t="n"/>
       <c r="K76" s="6" t="n"/>
       <c r="L76" s="2" t="n"/>
     </row>
-    <row r="77" ht="32" customHeight="1">
+    <row r="77">
       <c r="A77" s="2" t="n"/>
       <c r="B77" s="3" t="n"/>
       <c r="C77" s="4" t="n"/>
@@ -1613,11 +1616,11 @@
       <c r="G77" s="2" t="n"/>
       <c r="H77" s="2" t="n"/>
       <c r="I77" s="5" t="n"/>
-      <c r="J77" s="2" t="n"/>
+      <c r="J77" s="7" t="n"/>
       <c r="K77" s="6" t="n"/>
       <c r="L77" s="2" t="n"/>
     </row>
-    <row r="78" ht="32" customHeight="1">
+    <row r="78">
       <c r="A78" s="2" t="n"/>
       <c r="B78" s="3" t="n"/>
       <c r="C78" s="4" t="n"/>
@@ -1627,11 +1630,11 @@
       <c r="G78" s="2" t="n"/>
       <c r="H78" s="2" t="n"/>
       <c r="I78" s="5" t="n"/>
-      <c r="J78" s="2" t="n"/>
+      <c r="J78" s="7" t="n"/>
       <c r="K78" s="6" t="n"/>
       <c r="L78" s="2" t="n"/>
     </row>
-    <row r="79" ht="32" customHeight="1">
+    <row r="79">
       <c r="A79" s="2" t="n"/>
       <c r="B79" s="3" t="n"/>
       <c r="C79" s="4" t="n"/>
@@ -1641,11 +1644,11 @@
       <c r="G79" s="2" t="n"/>
       <c r="H79" s="2" t="n"/>
       <c r="I79" s="5" t="n"/>
-      <c r="J79" s="2" t="n"/>
+      <c r="J79" s="7" t="n"/>
       <c r="K79" s="6" t="n"/>
       <c r="L79" s="2" t="n"/>
     </row>
-    <row r="80" ht="32" customHeight="1">
+    <row r="80">
       <c r="A80" s="2" t="n"/>
       <c r="B80" s="3" t="n"/>
       <c r="C80" s="4" t="n"/>
@@ -1655,11 +1658,11 @@
       <c r="G80" s="2" t="n"/>
       <c r="H80" s="2" t="n"/>
       <c r="I80" s="5" t="n"/>
-      <c r="J80" s="2" t="n"/>
+      <c r="J80" s="7" t="n"/>
       <c r="K80" s="6" t="n"/>
       <c r="L80" s="2" t="n"/>
     </row>
-    <row r="81" ht="32" customHeight="1">
+    <row r="81">
       <c r="A81" s="2" t="n"/>
       <c r="B81" s="3" t="n"/>
       <c r="C81" s="4" t="n"/>
@@ -1669,11 +1672,11 @@
       <c r="G81" s="2" t="n"/>
       <c r="H81" s="2" t="n"/>
       <c r="I81" s="5" t="n"/>
-      <c r="J81" s="2" t="n"/>
+      <c r="J81" s="7" t="n"/>
       <c r="K81" s="6" t="n"/>
       <c r="L81" s="2" t="n"/>
     </row>
-    <row r="82" ht="32" customHeight="1">
+    <row r="82">
       <c r="A82" s="2" t="n"/>
       <c r="B82" s="3" t="n"/>
       <c r="C82" s="4" t="n"/>
@@ -1683,11 +1686,11 @@
       <c r="G82" s="2" t="n"/>
       <c r="H82" s="2" t="n"/>
       <c r="I82" s="5" t="n"/>
-      <c r="J82" s="2" t="n"/>
+      <c r="J82" s="7" t="n"/>
       <c r="K82" s="6" t="n"/>
       <c r="L82" s="2" t="n"/>
     </row>
-    <row r="83" ht="32" customHeight="1">
+    <row r="83">
       <c r="A83" s="2" t="n"/>
       <c r="B83" s="3" t="n"/>
       <c r="C83" s="4" t="n"/>
@@ -1697,11 +1700,11 @@
       <c r="G83" s="2" t="n"/>
       <c r="H83" s="2" t="n"/>
       <c r="I83" s="5" t="n"/>
-      <c r="J83" s="2" t="n"/>
+      <c r="J83" s="7" t="n"/>
       <c r="K83" s="6" t="n"/>
       <c r="L83" s="2" t="n"/>
     </row>
-    <row r="84" ht="32" customHeight="1">
+    <row r="84">
       <c r="A84" s="2" t="n"/>
       <c r="B84" s="3" t="n"/>
       <c r="C84" s="4" t="n"/>
@@ -1711,11 +1714,11 @@
       <c r="G84" s="2" t="n"/>
       <c r="H84" s="2" t="n"/>
       <c r="I84" s="5" t="n"/>
-      <c r="J84" s="2" t="n"/>
+      <c r="J84" s="7" t="n"/>
       <c r="K84" s="6" t="n"/>
       <c r="L84" s="2" t="n"/>
     </row>
-    <row r="85" ht="32" customHeight="1">
+    <row r="85">
       <c r="A85" s="2" t="n"/>
       <c r="B85" s="3" t="n"/>
       <c r="C85" s="4" t="n"/>
@@ -1725,11 +1728,11 @@
       <c r="G85" s="2" t="n"/>
       <c r="H85" s="2" t="n"/>
       <c r="I85" s="5" t="n"/>
-      <c r="J85" s="2" t="n"/>
+      <c r="J85" s="7" t="n"/>
       <c r="K85" s="6" t="n"/>
       <c r="L85" s="2" t="n"/>
     </row>
-    <row r="86" ht="32" customHeight="1">
+    <row r="86">
       <c r="A86" s="2" t="n"/>
       <c r="B86" s="3" t="n"/>
       <c r="C86" s="4" t="n"/>
@@ -1739,11 +1742,11 @@
       <c r="G86" s="2" t="n"/>
       <c r="H86" s="2" t="n"/>
       <c r="I86" s="5" t="n"/>
-      <c r="J86" s="2" t="n"/>
+      <c r="J86" s="7" t="n"/>
       <c r="K86" s="6" t="n"/>
       <c r="L86" s="2" t="n"/>
     </row>
-    <row r="87" ht="32" customHeight="1">
+    <row r="87">
       <c r="A87" s="2" t="n"/>
       <c r="B87" s="3" t="n"/>
       <c r="C87" s="4" t="n"/>
@@ -1753,11 +1756,11 @@
       <c r="G87" s="2" t="n"/>
       <c r="H87" s="2" t="n"/>
       <c r="I87" s="5" t="n"/>
-      <c r="J87" s="2" t="n"/>
+      <c r="J87" s="7" t="n"/>
       <c r="K87" s="6" t="n"/>
       <c r="L87" s="2" t="n"/>
     </row>
-    <row r="88" ht="32" customHeight="1">
+    <row r="88">
       <c r="A88" s="2" t="n"/>
       <c r="B88" s="3" t="n"/>
       <c r="C88" s="4" t="n"/>
@@ -1767,11 +1770,11 @@
       <c r="G88" s="2" t="n"/>
       <c r="H88" s="2" t="n"/>
       <c r="I88" s="5" t="n"/>
-      <c r="J88" s="2" t="n"/>
+      <c r="J88" s="7" t="n"/>
       <c r="K88" s="6" t="n"/>
       <c r="L88" s="2" t="n"/>
     </row>
-    <row r="89" ht="32" customHeight="1">
+    <row r="89">
       <c r="A89" s="2" t="n"/>
       <c r="B89" s="3" t="n"/>
       <c r="C89" s="4" t="n"/>
@@ -1781,11 +1784,11 @@
       <c r="G89" s="2" t="n"/>
       <c r="H89" s="2" t="n"/>
       <c r="I89" s="5" t="n"/>
-      <c r="J89" s="2" t="n"/>
+      <c r="J89" s="7" t="n"/>
       <c r="K89" s="6" t="n"/>
       <c r="L89" s="2" t="n"/>
     </row>
-    <row r="90" ht="32" customHeight="1">
+    <row r="90">
       <c r="A90" s="2" t="n"/>
       <c r="B90" s="3" t="n"/>
       <c r="C90" s="4" t="n"/>
@@ -1795,11 +1798,11 @@
       <c r="G90" s="2" t="n"/>
       <c r="H90" s="2" t="n"/>
       <c r="I90" s="5" t="n"/>
-      <c r="J90" s="2" t="n"/>
+      <c r="J90" s="7" t="n"/>
       <c r="K90" s="6" t="n"/>
       <c r="L90" s="2" t="n"/>
     </row>
-    <row r="91" ht="32" customHeight="1">
+    <row r="91">
       <c r="A91" s="2" t="n"/>
       <c r="B91" s="3" t="n"/>
       <c r="C91" s="4" t="n"/>
@@ -1809,11 +1812,11 @@
       <c r="G91" s="2" t="n"/>
       <c r="H91" s="2" t="n"/>
       <c r="I91" s="5" t="n"/>
-      <c r="J91" s="2" t="n"/>
+      <c r="J91" s="7" t="n"/>
       <c r="K91" s="6" t="n"/>
       <c r="L91" s="2" t="n"/>
     </row>
-    <row r="92" ht="32" customHeight="1">
+    <row r="92">
       <c r="A92" s="2" t="n"/>
       <c r="B92" s="3" t="n"/>
       <c r="C92" s="4" t="n"/>
@@ -1823,11 +1826,11 @@
       <c r="G92" s="2" t="n"/>
       <c r="H92" s="2" t="n"/>
       <c r="I92" s="5" t="n"/>
-      <c r="J92" s="2" t="n"/>
+      <c r="J92" s="7" t="n"/>
       <c r="K92" s="6" t="n"/>
       <c r="L92" s="2" t="n"/>
     </row>
-    <row r="93" ht="32" customHeight="1">
+    <row r="93">
       <c r="A93" s="2" t="n"/>
       <c r="B93" s="3" t="n"/>
       <c r="C93" s="4" t="n"/>
@@ -1837,11 +1840,11 @@
       <c r="G93" s="2" t="n"/>
       <c r="H93" s="2" t="n"/>
       <c r="I93" s="5" t="n"/>
-      <c r="J93" s="2" t="n"/>
+      <c r="J93" s="7" t="n"/>
       <c r="K93" s="6" t="n"/>
       <c r="L93" s="2" t="n"/>
     </row>
-    <row r="94" ht="32" customHeight="1">
+    <row r="94">
       <c r="A94" s="2" t="n"/>
       <c r="B94" s="3" t="n"/>
       <c r="C94" s="4" t="n"/>
@@ -1851,11 +1854,11 @@
       <c r="G94" s="2" t="n"/>
       <c r="H94" s="2" t="n"/>
       <c r="I94" s="5" t="n"/>
-      <c r="J94" s="2" t="n"/>
+      <c r="J94" s="7" t="n"/>
       <c r="K94" s="6" t="n"/>
       <c r="L94" s="2" t="n"/>
     </row>
-    <row r="95" ht="32" customHeight="1">
+    <row r="95">
       <c r="A95" s="2" t="n"/>
       <c r="B95" s="3" t="n"/>
       <c r="C95" s="4" t="n"/>
@@ -1865,11 +1868,11 @@
       <c r="G95" s="2" t="n"/>
       <c r="H95" s="2" t="n"/>
       <c r="I95" s="5" t="n"/>
-      <c r="J95" s="2" t="n"/>
+      <c r="J95" s="7" t="n"/>
       <c r="K95" s="6" t="n"/>
       <c r="L95" s="2" t="n"/>
     </row>
-    <row r="96" ht="32" customHeight="1">
+    <row r="96">
       <c r="A96" s="2" t="n"/>
       <c r="B96" s="3" t="n"/>
       <c r="C96" s="4" t="n"/>
@@ -1879,11 +1882,11 @@
       <c r="G96" s="2" t="n"/>
       <c r="H96" s="2" t="n"/>
       <c r="I96" s="5" t="n"/>
-      <c r="J96" s="2" t="n"/>
+      <c r="J96" s="7" t="n"/>
       <c r="K96" s="6" t="n"/>
       <c r="L96" s="2" t="n"/>
     </row>
-    <row r="97" ht="32" customHeight="1">
+    <row r="97">
       <c r="A97" s="2" t="n"/>
       <c r="B97" s="3" t="n"/>
       <c r="C97" s="4" t="n"/>
@@ -1893,11 +1896,11 @@
       <c r="G97" s="2" t="n"/>
       <c r="H97" s="2" t="n"/>
       <c r="I97" s="5" t="n"/>
-      <c r="J97" s="2" t="n"/>
+      <c r="J97" s="7" t="n"/>
       <c r="K97" s="6" t="n"/>
       <c r="L97" s="2" t="n"/>
     </row>
-    <row r="98" ht="32" customHeight="1">
+    <row r="98">
       <c r="A98" s="2" t="n"/>
       <c r="B98" s="3" t="n"/>
       <c r="C98" s="4" t="n"/>
@@ -1907,11 +1910,11 @@
       <c r="G98" s="2" t="n"/>
       <c r="H98" s="2" t="n"/>
       <c r="I98" s="5" t="n"/>
-      <c r="J98" s="2" t="n"/>
+      <c r="J98" s="7" t="n"/>
       <c r="K98" s="6" t="n"/>
       <c r="L98" s="2" t="n"/>
     </row>
-    <row r="99" ht="32" customHeight="1">
+    <row r="99">
       <c r="A99" s="2" t="n"/>
       <c r="B99" s="3" t="n"/>
       <c r="C99" s="4" t="n"/>
@@ -1921,11 +1924,11 @@
       <c r="G99" s="2" t="n"/>
       <c r="H99" s="2" t="n"/>
       <c r="I99" s="5" t="n"/>
-      <c r="J99" s="2" t="n"/>
+      <c r="J99" s="7" t="n"/>
       <c r="K99" s="6" t="n"/>
       <c r="L99" s="2" t="n"/>
     </row>
-    <row r="100" ht="32" customHeight="1">
+    <row r="100">
       <c r="A100" s="2" t="n"/>
       <c r="B100" s="3" t="n"/>
       <c r="C100" s="4" t="n"/>
@@ -1935,11 +1938,11 @@
       <c r="G100" s="2" t="n"/>
       <c r="H100" s="2" t="n"/>
       <c r="I100" s="5" t="n"/>
-      <c r="J100" s="2" t="n"/>
+      <c r="J100" s="7" t="n"/>
       <c r="K100" s="6" t="n"/>
       <c r="L100" s="2" t="n"/>
     </row>
-    <row r="101" ht="32" customHeight="1">
+    <row r="101">
       <c r="A101" s="2" t="n"/>
       <c r="B101" s="3" t="n"/>
       <c r="C101" s="4" t="n"/>
@@ -1949,7 +1952,7 @@
       <c r="G101" s="2" t="n"/>
       <c r="H101" s="2" t="n"/>
       <c r="I101" s="5" t="n"/>
-      <c r="J101" s="2" t="n"/>
+      <c r="J101" s="7" t="n"/>
       <c r="K101" s="6" t="n"/>
       <c r="L101" s="2" t="n"/>
     </row>

</xml_diff>